<commit_message>
Fix double-counted September; add full-year totals to best/worst workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/المستهدف_الشهري_أفضل_أسوأ.xlsx
+++ b/المستهدف_الشهري_أفضل_أسوأ.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AF49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,10 @@
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,7 +531,7 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأفضل: لكل شهر، الأكبر بين التوقع الأساسي ومتوسط أعلى قيمتين تاريخيتين لنفس الشهر (2023–2025) × معامل الاتجاه (لا يقل عن 1)، بسقف 1.5 ضعف الأساسي.</t>
+          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأفضل: لكل شهر، الأكبر بين التوقع الأساسي ومتوسط أعلى قيمتين تاريخيتين لنفس الشهر (2023–2025) × معامل الاتجاه (لا يقل عن 1)، بسقف 1.5 ضعف الأساسي.</t>
         </is>
       </c>
     </row>
@@ -557,7 +561,7 @@
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>سبتمبر (فعلي)</t>
+          <t>منها سبتمبر (مشمول في التراكمي، لا يُجمع معه)</t>
         </is>
       </c>
       <c r="I4" s="3" t="n"/>
@@ -590,12 +594,20 @@
       <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>المجموع سبتمبر–ديسمبر</t>
+          <t>المجموع أكتوبر–ديسمبر</t>
         </is>
       </c>
       <c r="Z4" s="3" t="n"/>
       <c r="AA4" s="3" t="n"/>
       <c r="AB4" s="3" t="n"/>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>إجمالي السنة 2026 (يناير–ديسمبر)</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="n"/>
+      <c r="AE4" s="3" t="n"/>
+      <c r="AF4" s="3" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="3" t="n"/>
@@ -713,7 +725,7 @@
       </c>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>المحصل + المتوقع</t>
+          <t>المتوقع</t>
         </is>
       </c>
       <c r="AA5" s="3" t="inlineStr">
@@ -722,6 +734,26 @@
         </is>
       </c>
       <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف السنوي</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل الفعلي + المتوقع</t>
+        </is>
+      </c>
+      <c r="AE5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="AF5" s="3" t="inlineStr">
         <is>
           <t>% من المستهدف</t>
         </is>
@@ -824,11 +856,11 @@
         <v/>
       </c>
       <c r="Y6" s="5">
-        <f>H6+L6+Q6+U6</f>
+        <f>L6+Q6+U6</f>
         <v/>
       </c>
       <c r="Z6" s="5">
-        <f>I6+N6+R6+V6</f>
+        <f>N6+R6+V6</f>
         <v/>
       </c>
       <c r="AA6" s="5">
@@ -837,6 +869,22 @@
       </c>
       <c r="AB6" s="6">
         <f>IF(Y6=0,"",Z6/Y6)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="5">
+        <f>D6+Y6</f>
+        <v/>
+      </c>
+      <c r="AD6" s="5">
+        <f>E6+Z6</f>
+        <v/>
+      </c>
+      <c r="AE6" s="5">
+        <f>AD6-AC6</f>
+        <v/>
+      </c>
+      <c r="AF6" s="6">
+        <f>IF(AC6=0,"",AD6/AC6)</f>
         <v/>
       </c>
     </row>
@@ -930,11 +978,11 @@
         <v/>
       </c>
       <c r="Y7" s="8">
-        <f>H7+L7+Q7+U7</f>
+        <f>L7+Q7+U7</f>
         <v/>
       </c>
       <c r="Z7" s="8">
-        <f>I7+N7+R7+V7</f>
+        <f>N7+R7+V7</f>
         <v/>
       </c>
       <c r="AA7" s="8">
@@ -943,6 +991,22 @@
       </c>
       <c r="AB7" s="9">
         <f>IF(Y7=0,"",Z7/Y7)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="8">
+        <f>D7+Y7</f>
+        <v/>
+      </c>
+      <c r="AD7" s="8">
+        <f>E7+Z7</f>
+        <v/>
+      </c>
+      <c r="AE7" s="8">
+        <f>AD7-AC7</f>
+        <v/>
+      </c>
+      <c r="AF7" s="9">
+        <f>IF(AC7=0,"",AD7/AC7)</f>
         <v/>
       </c>
     </row>
@@ -1036,11 +1100,11 @@
         <v/>
       </c>
       <c r="Y8" s="8">
-        <f>H8+L8+Q8+U8</f>
+        <f>L8+Q8+U8</f>
         <v/>
       </c>
       <c r="Z8" s="8">
-        <f>I8+N8+R8+V8</f>
+        <f>N8+R8+V8</f>
         <v/>
       </c>
       <c r="AA8" s="8">
@@ -1049,6 +1113,22 @@
       </c>
       <c r="AB8" s="9">
         <f>IF(Y8=0,"",Z8/Y8)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="8">
+        <f>D8+Y8</f>
+        <v/>
+      </c>
+      <c r="AD8" s="8">
+        <f>E8+Z8</f>
+        <v/>
+      </c>
+      <c r="AE8" s="8">
+        <f>AD8-AC8</f>
+        <v/>
+      </c>
+      <c r="AF8" s="9">
+        <f>IF(AC8=0,"",AD8/AC8)</f>
         <v/>
       </c>
     </row>
@@ -1142,11 +1222,11 @@
         <v/>
       </c>
       <c r="Y9" s="8">
-        <f>H9+L9+Q9+U9</f>
+        <f>L9+Q9+U9</f>
         <v/>
       </c>
       <c r="Z9" s="8">
-        <f>I9+N9+R9+V9</f>
+        <f>N9+R9+V9</f>
         <v/>
       </c>
       <c r="AA9" s="8">
@@ -1155,6 +1235,22 @@
       </c>
       <c r="AB9" s="9">
         <f>IF(Y9=0,"",Z9/Y9)</f>
+        <v/>
+      </c>
+      <c r="AC9" s="8">
+        <f>D9+Y9</f>
+        <v/>
+      </c>
+      <c r="AD9" s="8">
+        <f>E9+Z9</f>
+        <v/>
+      </c>
+      <c r="AE9" s="8">
+        <f>AD9-AC9</f>
+        <v/>
+      </c>
+      <c r="AF9" s="9">
+        <f>IF(AC9=0,"",AD9/AC9)</f>
         <v/>
       </c>
     </row>
@@ -1248,11 +1344,11 @@
         <v/>
       </c>
       <c r="Y10" s="8">
-        <f>H10+L10+Q10+U10</f>
+        <f>L10+Q10+U10</f>
         <v/>
       </c>
       <c r="Z10" s="8">
-        <f>I10+N10+R10+V10</f>
+        <f>N10+R10+V10</f>
         <v/>
       </c>
       <c r="AA10" s="8">
@@ -1261,6 +1357,22 @@
       </c>
       <c r="AB10" s="9">
         <f>IF(Y10=0,"",Z10/Y10)</f>
+        <v/>
+      </c>
+      <c r="AC10" s="8">
+        <f>D10+Y10</f>
+        <v/>
+      </c>
+      <c r="AD10" s="8">
+        <f>E10+Z10</f>
+        <v/>
+      </c>
+      <c r="AE10" s="8">
+        <f>AD10-AC10</f>
+        <v/>
+      </c>
+      <c r="AF10" s="9">
+        <f>IF(AC10=0,"",AD10/AC10)</f>
         <v/>
       </c>
     </row>
@@ -1354,11 +1466,11 @@
         <v/>
       </c>
       <c r="Y11" s="8">
-        <f>H11+L11+Q11+U11</f>
+        <f>L11+Q11+U11</f>
         <v/>
       </c>
       <c r="Z11" s="8">
-        <f>I11+N11+R11+V11</f>
+        <f>N11+R11+V11</f>
         <v/>
       </c>
       <c r="AA11" s="8">
@@ -1367,6 +1479,22 @@
       </c>
       <c r="AB11" s="9">
         <f>IF(Y11=0,"",Z11/Y11)</f>
+        <v/>
+      </c>
+      <c r="AC11" s="8">
+        <f>D11+Y11</f>
+        <v/>
+      </c>
+      <c r="AD11" s="8">
+        <f>E11+Z11</f>
+        <v/>
+      </c>
+      <c r="AE11" s="8">
+        <f>AD11-AC11</f>
+        <v/>
+      </c>
+      <c r="AF11" s="9">
+        <f>IF(AC11=0,"",AD11/AC11)</f>
         <v/>
       </c>
     </row>
@@ -1460,11 +1588,11 @@
         <v/>
       </c>
       <c r="Y12" s="8">
-        <f>H12+L12+Q12+U12</f>
+        <f>L12+Q12+U12</f>
         <v/>
       </c>
       <c r="Z12" s="8">
-        <f>I12+N12+R12+V12</f>
+        <f>N12+R12+V12</f>
         <v/>
       </c>
       <c r="AA12" s="8">
@@ -1473,6 +1601,22 @@
       </c>
       <c r="AB12" s="9">
         <f>IF(Y12=0,"",Z12/Y12)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="8">
+        <f>D12+Y12</f>
+        <v/>
+      </c>
+      <c r="AD12" s="8">
+        <f>E12+Z12</f>
+        <v/>
+      </c>
+      <c r="AE12" s="8">
+        <f>AD12-AC12</f>
+        <v/>
+      </c>
+      <c r="AF12" s="9">
+        <f>IF(AC12=0,"",AD12/AC12)</f>
         <v/>
       </c>
     </row>
@@ -1566,11 +1710,11 @@
         <v/>
       </c>
       <c r="Y13" s="8">
-        <f>H13+L13+Q13+U13</f>
+        <f>L13+Q13+U13</f>
         <v/>
       </c>
       <c r="Z13" s="8">
-        <f>I13+N13+R13+V13</f>
+        <f>N13+R13+V13</f>
         <v/>
       </c>
       <c r="AA13" s="8">
@@ -1579,6 +1723,22 @@
       </c>
       <c r="AB13" s="9">
         <f>IF(Y13=0,"",Z13/Y13)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="8">
+        <f>D13+Y13</f>
+        <v/>
+      </c>
+      <c r="AD13" s="8">
+        <f>E13+Z13</f>
+        <v/>
+      </c>
+      <c r="AE13" s="8">
+        <f>AD13-AC13</f>
+        <v/>
+      </c>
+      <c r="AF13" s="9">
+        <f>IF(AC13=0,"",AD13/AC13)</f>
         <v/>
       </c>
     </row>
@@ -1679,11 +1839,11 @@
         <v/>
       </c>
       <c r="Y14" s="5">
-        <f>H14+L14+Q14+U14</f>
+        <f>L14+Q14+U14</f>
         <v/>
       </c>
       <c r="Z14" s="5">
-        <f>I14+N14+R14+V14</f>
+        <f>N14+R14+V14</f>
         <v/>
       </c>
       <c r="AA14" s="5">
@@ -1692,6 +1852,22 @@
       </c>
       <c r="AB14" s="6">
         <f>IF(Y14=0,"",Z14/Y14)</f>
+        <v/>
+      </c>
+      <c r="AC14" s="5">
+        <f>D14+Y14</f>
+        <v/>
+      </c>
+      <c r="AD14" s="5">
+        <f>E14+Z14</f>
+        <v/>
+      </c>
+      <c r="AE14" s="5">
+        <f>AD14-AC14</f>
+        <v/>
+      </c>
+      <c r="AF14" s="6">
+        <f>IF(AC14=0,"",AD14/AC14)</f>
         <v/>
       </c>
     </row>
@@ -1785,11 +1961,11 @@
         <v/>
       </c>
       <c r="Y15" s="8">
-        <f>H15+L15+Q15+U15</f>
+        <f>L15+Q15+U15</f>
         <v/>
       </c>
       <c r="Z15" s="8">
-        <f>I15+N15+R15+V15</f>
+        <f>N15+R15+V15</f>
         <v/>
       </c>
       <c r="AA15" s="8">
@@ -1798,6 +1974,22 @@
       </c>
       <c r="AB15" s="9">
         <f>IF(Y15=0,"",Z15/Y15)</f>
+        <v/>
+      </c>
+      <c r="AC15" s="8">
+        <f>D15+Y15</f>
+        <v/>
+      </c>
+      <c r="AD15" s="8">
+        <f>E15+Z15</f>
+        <v/>
+      </c>
+      <c r="AE15" s="8">
+        <f>AD15-AC15</f>
+        <v/>
+      </c>
+      <c r="AF15" s="9">
+        <f>IF(AC15=0,"",AD15/AC15)</f>
         <v/>
       </c>
     </row>
@@ -1891,11 +2083,11 @@
         <v/>
       </c>
       <c r="Y16" s="8">
-        <f>H16+L16+Q16+U16</f>
+        <f>L16+Q16+U16</f>
         <v/>
       </c>
       <c r="Z16" s="8">
-        <f>I16+N16+R16+V16</f>
+        <f>N16+R16+V16</f>
         <v/>
       </c>
       <c r="AA16" s="8">
@@ -1904,6 +2096,22 @@
       </c>
       <c r="AB16" s="9">
         <f>IF(Y16=0,"",Z16/Y16)</f>
+        <v/>
+      </c>
+      <c r="AC16" s="8">
+        <f>D16+Y16</f>
+        <v/>
+      </c>
+      <c r="AD16" s="8">
+        <f>E16+Z16</f>
+        <v/>
+      </c>
+      <c r="AE16" s="8">
+        <f>AD16-AC16</f>
+        <v/>
+      </c>
+      <c r="AF16" s="9">
+        <f>IF(AC16=0,"",AD16/AC16)</f>
         <v/>
       </c>
     </row>
@@ -1997,11 +2205,11 @@
         <v/>
       </c>
       <c r="Y17" s="8">
-        <f>H17+L17+Q17+U17</f>
+        <f>L17+Q17+U17</f>
         <v/>
       </c>
       <c r="Z17" s="8">
-        <f>I17+N17+R17+V17</f>
+        <f>N17+R17+V17</f>
         <v/>
       </c>
       <c r="AA17" s="8">
@@ -2010,6 +2218,22 @@
       </c>
       <c r="AB17" s="9">
         <f>IF(Y17=0,"",Z17/Y17)</f>
+        <v/>
+      </c>
+      <c r="AC17" s="8">
+        <f>D17+Y17</f>
+        <v/>
+      </c>
+      <c r="AD17" s="8">
+        <f>E17+Z17</f>
+        <v/>
+      </c>
+      <c r="AE17" s="8">
+        <f>AD17-AC17</f>
+        <v/>
+      </c>
+      <c r="AF17" s="9">
+        <f>IF(AC17=0,"",AD17/AC17)</f>
         <v/>
       </c>
     </row>
@@ -2103,11 +2327,11 @@
         <v/>
       </c>
       <c r="Y18" s="8">
-        <f>H18+L18+Q18+U18</f>
+        <f>L18+Q18+U18</f>
         <v/>
       </c>
       <c r="Z18" s="8">
-        <f>I18+N18+R18+V18</f>
+        <f>N18+R18+V18</f>
         <v/>
       </c>
       <c r="AA18" s="8">
@@ -2116,6 +2340,22 @@
       </c>
       <c r="AB18" s="9">
         <f>IF(Y18=0,"",Z18/Y18)</f>
+        <v/>
+      </c>
+      <c r="AC18" s="8">
+        <f>D18+Y18</f>
+        <v/>
+      </c>
+      <c r="AD18" s="8">
+        <f>E18+Z18</f>
+        <v/>
+      </c>
+      <c r="AE18" s="8">
+        <f>AD18-AC18</f>
+        <v/>
+      </c>
+      <c r="AF18" s="9">
+        <f>IF(AC18=0,"",AD18/AC18)</f>
         <v/>
       </c>
     </row>
@@ -2209,11 +2449,11 @@
         <v/>
       </c>
       <c r="Y19" s="8">
-        <f>H19+L19+Q19+U19</f>
+        <f>L19+Q19+U19</f>
         <v/>
       </c>
       <c r="Z19" s="8">
-        <f>I19+N19+R19+V19</f>
+        <f>N19+R19+V19</f>
         <v/>
       </c>
       <c r="AA19" s="8">
@@ -2222,6 +2462,22 @@
       </c>
       <c r="AB19" s="9">
         <f>IF(Y19=0,"",Z19/Y19)</f>
+        <v/>
+      </c>
+      <c r="AC19" s="8">
+        <f>D19+Y19</f>
+        <v/>
+      </c>
+      <c r="AD19" s="8">
+        <f>E19+Z19</f>
+        <v/>
+      </c>
+      <c r="AE19" s="8">
+        <f>AD19-AC19</f>
+        <v/>
+      </c>
+      <c r="AF19" s="9">
+        <f>IF(AC19=0,"",AD19/AC19)</f>
         <v/>
       </c>
     </row>
@@ -2315,11 +2571,11 @@
         <v/>
       </c>
       <c r="Y20" s="8">
-        <f>H20+L20+Q20+U20</f>
+        <f>L20+Q20+U20</f>
         <v/>
       </c>
       <c r="Z20" s="8">
-        <f>I20+N20+R20+V20</f>
+        <f>N20+R20+V20</f>
         <v/>
       </c>
       <c r="AA20" s="8">
@@ -2328,6 +2584,22 @@
       </c>
       <c r="AB20" s="9">
         <f>IF(Y20=0,"",Z20/Y20)</f>
+        <v/>
+      </c>
+      <c r="AC20" s="8">
+        <f>D20+Y20</f>
+        <v/>
+      </c>
+      <c r="AD20" s="8">
+        <f>E20+Z20</f>
+        <v/>
+      </c>
+      <c r="AE20" s="8">
+        <f>AD20-AC20</f>
+        <v/>
+      </c>
+      <c r="AF20" s="9">
+        <f>IF(AC20=0,"",AD20/AC20)</f>
         <v/>
       </c>
     </row>
@@ -2421,11 +2693,11 @@
         <v/>
       </c>
       <c r="Y21" s="8">
-        <f>H21+L21+Q21+U21</f>
+        <f>L21+Q21+U21</f>
         <v/>
       </c>
       <c r="Z21" s="8">
-        <f>I21+N21+R21+V21</f>
+        <f>N21+R21+V21</f>
         <v/>
       </c>
       <c r="AA21" s="8">
@@ -2434,6 +2706,22 @@
       </c>
       <c r="AB21" s="9">
         <f>IF(Y21=0,"",Z21/Y21)</f>
+        <v/>
+      </c>
+      <c r="AC21" s="8">
+        <f>D21+Y21</f>
+        <v/>
+      </c>
+      <c r="AD21" s="8">
+        <f>E21+Z21</f>
+        <v/>
+      </c>
+      <c r="AE21" s="8">
+        <f>AD21-AC21</f>
+        <v/>
+      </c>
+      <c r="AF21" s="9">
+        <f>IF(AC21=0,"",AD21/AC21)</f>
         <v/>
       </c>
     </row>
@@ -2527,11 +2815,11 @@
         <v/>
       </c>
       <c r="Y22" s="8">
-        <f>H22+L22+Q22+U22</f>
+        <f>L22+Q22+U22</f>
         <v/>
       </c>
       <c r="Z22" s="8">
-        <f>I22+N22+R22+V22</f>
+        <f>N22+R22+V22</f>
         <v/>
       </c>
       <c r="AA22" s="8">
@@ -2540,6 +2828,22 @@
       </c>
       <c r="AB22" s="9">
         <f>IF(Y22=0,"",Z22/Y22)</f>
+        <v/>
+      </c>
+      <c r="AC22" s="8">
+        <f>D22+Y22</f>
+        <v/>
+      </c>
+      <c r="AD22" s="8">
+        <f>E22+Z22</f>
+        <v/>
+      </c>
+      <c r="AE22" s="8">
+        <f>AD22-AC22</f>
+        <v/>
+      </c>
+      <c r="AF22" s="9">
+        <f>IF(AC22=0,"",AD22/AC22)</f>
         <v/>
       </c>
     </row>
@@ -2633,11 +2937,11 @@
         <v/>
       </c>
       <c r="Y23" s="8">
-        <f>H23+L23+Q23+U23</f>
+        <f>L23+Q23+U23</f>
         <v/>
       </c>
       <c r="Z23" s="8">
-        <f>I23+N23+R23+V23</f>
+        <f>N23+R23+V23</f>
         <v/>
       </c>
       <c r="AA23" s="8">
@@ -2646,6 +2950,22 @@
       </c>
       <c r="AB23" s="9">
         <f>IF(Y23=0,"",Z23/Y23)</f>
+        <v/>
+      </c>
+      <c r="AC23" s="8">
+        <f>D23+Y23</f>
+        <v/>
+      </c>
+      <c r="AD23" s="8">
+        <f>E23+Z23</f>
+        <v/>
+      </c>
+      <c r="AE23" s="8">
+        <f>AD23-AC23</f>
+        <v/>
+      </c>
+      <c r="AF23" s="9">
+        <f>IF(AC23=0,"",AD23/AC23)</f>
         <v/>
       </c>
     </row>
@@ -2739,11 +3059,11 @@
         <v/>
       </c>
       <c r="Y24" s="8">
-        <f>H24+L24+Q24+U24</f>
+        <f>L24+Q24+U24</f>
         <v/>
       </c>
       <c r="Z24" s="8">
-        <f>I24+N24+R24+V24</f>
+        <f>N24+R24+V24</f>
         <v/>
       </c>
       <c r="AA24" s="8">
@@ -2752,6 +3072,22 @@
       </c>
       <c r="AB24" s="9">
         <f>IF(Y24=0,"",Z24/Y24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="8">
+        <f>D24+Y24</f>
+        <v/>
+      </c>
+      <c r="AD24" s="8">
+        <f>E24+Z24</f>
+        <v/>
+      </c>
+      <c r="AE24" s="8">
+        <f>AD24-AC24</f>
+        <v/>
+      </c>
+      <c r="AF24" s="9">
+        <f>IF(AC24=0,"",AD24/AC24)</f>
         <v/>
       </c>
     </row>
@@ -2845,11 +3181,11 @@
         <v/>
       </c>
       <c r="Y25" s="8">
-        <f>H25+L25+Q25+U25</f>
+        <f>L25+Q25+U25</f>
         <v/>
       </c>
       <c r="Z25" s="8">
-        <f>I25+N25+R25+V25</f>
+        <f>N25+R25+V25</f>
         <v/>
       </c>
       <c r="AA25" s="8">
@@ -2858,6 +3194,22 @@
       </c>
       <c r="AB25" s="9">
         <f>IF(Y25=0,"",Z25/Y25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="8">
+        <f>D25+Y25</f>
+        <v/>
+      </c>
+      <c r="AD25" s="8">
+        <f>E25+Z25</f>
+        <v/>
+      </c>
+      <c r="AE25" s="8">
+        <f>AD25-AC25</f>
+        <v/>
+      </c>
+      <c r="AF25" s="9">
+        <f>IF(AC25=0,"",AD25/AC25)</f>
         <v/>
       </c>
     </row>
@@ -2951,11 +3303,11 @@
         <v/>
       </c>
       <c r="Y26" s="8">
-        <f>H26+L26+Q26+U26</f>
+        <f>L26+Q26+U26</f>
         <v/>
       </c>
       <c r="Z26" s="8">
-        <f>I26+N26+R26+V26</f>
+        <f>N26+R26+V26</f>
         <v/>
       </c>
       <c r="AA26" s="8">
@@ -2964,6 +3316,22 @@
       </c>
       <c r="AB26" s="9">
         <f>IF(Y26=0,"",Z26/Y26)</f>
+        <v/>
+      </c>
+      <c r="AC26" s="8">
+        <f>D26+Y26</f>
+        <v/>
+      </c>
+      <c r="AD26" s="8">
+        <f>E26+Z26</f>
+        <v/>
+      </c>
+      <c r="AE26" s="8">
+        <f>AD26-AC26</f>
+        <v/>
+      </c>
+      <c r="AF26" s="9">
+        <f>IF(AC26=0,"",AD26/AC26)</f>
         <v/>
       </c>
     </row>
@@ -3057,11 +3425,11 @@
         <v/>
       </c>
       <c r="Y27" s="8">
-        <f>H27+L27+Q27+U27</f>
+        <f>L27+Q27+U27</f>
         <v/>
       </c>
       <c r="Z27" s="8">
-        <f>I27+N27+R27+V27</f>
+        <f>N27+R27+V27</f>
         <v/>
       </c>
       <c r="AA27" s="8">
@@ -3070,6 +3438,22 @@
       </c>
       <c r="AB27" s="9">
         <f>IF(Y27=0,"",Z27/Y27)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="8">
+        <f>D27+Y27</f>
+        <v/>
+      </c>
+      <c r="AD27" s="8">
+        <f>E27+Z27</f>
+        <v/>
+      </c>
+      <c r="AE27" s="8">
+        <f>AD27-AC27</f>
+        <v/>
+      </c>
+      <c r="AF27" s="9">
+        <f>IF(AC27=0,"",AD27/AC27)</f>
         <v/>
       </c>
     </row>
@@ -3163,11 +3547,11 @@
         <v/>
       </c>
       <c r="Y28" s="8">
-        <f>H28+L28+Q28+U28</f>
+        <f>L28+Q28+U28</f>
         <v/>
       </c>
       <c r="Z28" s="8">
-        <f>I28+N28+R28+V28</f>
+        <f>N28+R28+V28</f>
         <v/>
       </c>
       <c r="AA28" s="8">
@@ -3176,6 +3560,22 @@
       </c>
       <c r="AB28" s="9">
         <f>IF(Y28=0,"",Z28/Y28)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="8">
+        <f>D28+Y28</f>
+        <v/>
+      </c>
+      <c r="AD28" s="8">
+        <f>E28+Z28</f>
+        <v/>
+      </c>
+      <c r="AE28" s="8">
+        <f>AD28-AC28</f>
+        <v/>
+      </c>
+      <c r="AF28" s="9">
+        <f>IF(AC28=0,"",AD28/AC28)</f>
         <v/>
       </c>
     </row>
@@ -3269,11 +3669,11 @@
         <v/>
       </c>
       <c r="Y29" s="8">
-        <f>H29+L29+Q29+U29</f>
+        <f>L29+Q29+U29</f>
         <v/>
       </c>
       <c r="Z29" s="8">
-        <f>I29+N29+R29+V29</f>
+        <f>N29+R29+V29</f>
         <v/>
       </c>
       <c r="AA29" s="8">
@@ -3282,6 +3682,22 @@
       </c>
       <c r="AB29" s="9">
         <f>IF(Y29=0,"",Z29/Y29)</f>
+        <v/>
+      </c>
+      <c r="AC29" s="8">
+        <f>D29+Y29</f>
+        <v/>
+      </c>
+      <c r="AD29" s="8">
+        <f>E29+Z29</f>
+        <v/>
+      </c>
+      <c r="AE29" s="8">
+        <f>AD29-AC29</f>
+        <v/>
+      </c>
+      <c r="AF29" s="9">
+        <f>IF(AC29=0,"",AD29/AC29)</f>
         <v/>
       </c>
     </row>
@@ -3375,11 +3791,11 @@
         <v/>
       </c>
       <c r="Y30" s="8">
-        <f>H30+L30+Q30+U30</f>
+        <f>L30+Q30+U30</f>
         <v/>
       </c>
       <c r="Z30" s="8">
-        <f>I30+N30+R30+V30</f>
+        <f>N30+R30+V30</f>
         <v/>
       </c>
       <c r="AA30" s="8">
@@ -3388,6 +3804,22 @@
       </c>
       <c r="AB30" s="9">
         <f>IF(Y30=0,"",Z30/Y30)</f>
+        <v/>
+      </c>
+      <c r="AC30" s="8">
+        <f>D30+Y30</f>
+        <v/>
+      </c>
+      <c r="AD30" s="8">
+        <f>E30+Z30</f>
+        <v/>
+      </c>
+      <c r="AE30" s="8">
+        <f>AD30-AC30</f>
+        <v/>
+      </c>
+      <c r="AF30" s="9">
+        <f>IF(AC30=0,"",AD30/AC30)</f>
         <v/>
       </c>
     </row>
@@ -3481,11 +3913,11 @@
         <v/>
       </c>
       <c r="Y31" s="8">
-        <f>H31+L31+Q31+U31</f>
+        <f>L31+Q31+U31</f>
         <v/>
       </c>
       <c r="Z31" s="8">
-        <f>I31+N31+R31+V31</f>
+        <f>N31+R31+V31</f>
         <v/>
       </c>
       <c r="AA31" s="8">
@@ -3494,6 +3926,22 @@
       </c>
       <c r="AB31" s="9">
         <f>IF(Y31=0,"",Z31/Y31)</f>
+        <v/>
+      </c>
+      <c r="AC31" s="8">
+        <f>D31+Y31</f>
+        <v/>
+      </c>
+      <c r="AD31" s="8">
+        <f>E31+Z31</f>
+        <v/>
+      </c>
+      <c r="AE31" s="8">
+        <f>AD31-AC31</f>
+        <v/>
+      </c>
+      <c r="AF31" s="9">
+        <f>IF(AC31=0,"",AD31/AC31)</f>
         <v/>
       </c>
     </row>
@@ -3587,11 +4035,11 @@
         <v/>
       </c>
       <c r="Y32" s="8">
-        <f>H32+L32+Q32+U32</f>
+        <f>L32+Q32+U32</f>
         <v/>
       </c>
       <c r="Z32" s="8">
-        <f>I32+N32+R32+V32</f>
+        <f>N32+R32+V32</f>
         <v/>
       </c>
       <c r="AA32" s="8">
@@ -3600,6 +4048,22 @@
       </c>
       <c r="AB32" s="9">
         <f>IF(Y32=0,"",Z32/Y32)</f>
+        <v/>
+      </c>
+      <c r="AC32" s="8">
+        <f>D32+Y32</f>
+        <v/>
+      </c>
+      <c r="AD32" s="8">
+        <f>E32+Z32</f>
+        <v/>
+      </c>
+      <c r="AE32" s="8">
+        <f>AD32-AC32</f>
+        <v/>
+      </c>
+      <c r="AF32" s="9">
+        <f>IF(AC32=0,"",AD32/AC32)</f>
         <v/>
       </c>
     </row>
@@ -3700,11 +4164,11 @@
         <v/>
       </c>
       <c r="Y33" s="5">
-        <f>H33+L33+Q33+U33</f>
+        <f>L33+Q33+U33</f>
         <v/>
       </c>
       <c r="Z33" s="5">
-        <f>I33+N33+R33+V33</f>
+        <f>N33+R33+V33</f>
         <v/>
       </c>
       <c r="AA33" s="5">
@@ -3713,6 +4177,22 @@
       </c>
       <c r="AB33" s="6">
         <f>IF(Y33=0,"",Z33/Y33)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="5">
+        <f>D33+Y33</f>
+        <v/>
+      </c>
+      <c r="AD33" s="5">
+        <f>E33+Z33</f>
+        <v/>
+      </c>
+      <c r="AE33" s="5">
+        <f>AD33-AC33</f>
+        <v/>
+      </c>
+      <c r="AF33" s="6">
+        <f>IF(AC33=0,"",AD33/AC33)</f>
         <v/>
       </c>
     </row>
@@ -3806,11 +4286,11 @@
         <v/>
       </c>
       <c r="Y34" s="8">
-        <f>H34+L34+Q34+U34</f>
+        <f>L34+Q34+U34</f>
         <v/>
       </c>
       <c r="Z34" s="8">
-        <f>I34+N34+R34+V34</f>
+        <f>N34+R34+V34</f>
         <v/>
       </c>
       <c r="AA34" s="8">
@@ -3819,6 +4299,22 @@
       </c>
       <c r="AB34" s="9">
         <f>IF(Y34=0,"",Z34/Y34)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="8">
+        <f>D34+Y34</f>
+        <v/>
+      </c>
+      <c r="AD34" s="8">
+        <f>E34+Z34</f>
+        <v/>
+      </c>
+      <c r="AE34" s="8">
+        <f>AD34-AC34</f>
+        <v/>
+      </c>
+      <c r="AF34" s="9">
+        <f>IF(AC34=0,"",AD34/AC34)</f>
         <v/>
       </c>
     </row>
@@ -3912,11 +4408,11 @@
         <v/>
       </c>
       <c r="Y35" s="8">
-        <f>H35+L35+Q35+U35</f>
+        <f>L35+Q35+U35</f>
         <v/>
       </c>
       <c r="Z35" s="8">
-        <f>I35+N35+R35+V35</f>
+        <f>N35+R35+V35</f>
         <v/>
       </c>
       <c r="AA35" s="8">
@@ -3925,6 +4421,22 @@
       </c>
       <c r="AB35" s="9">
         <f>IF(Y35=0,"",Z35/Y35)</f>
+        <v/>
+      </c>
+      <c r="AC35" s="8">
+        <f>D35+Y35</f>
+        <v/>
+      </c>
+      <c r="AD35" s="8">
+        <f>E35+Z35</f>
+        <v/>
+      </c>
+      <c r="AE35" s="8">
+        <f>AD35-AC35</f>
+        <v/>
+      </c>
+      <c r="AF35" s="9">
+        <f>IF(AC35=0,"",AD35/AC35)</f>
         <v/>
       </c>
     </row>
@@ -4018,11 +4530,11 @@
         <v/>
       </c>
       <c r="Y36" s="8">
-        <f>H36+L36+Q36+U36</f>
+        <f>L36+Q36+U36</f>
         <v/>
       </c>
       <c r="Z36" s="8">
-        <f>I36+N36+R36+V36</f>
+        <f>N36+R36+V36</f>
         <v/>
       </c>
       <c r="AA36" s="8">
@@ -4031,6 +4543,22 @@
       </c>
       <c r="AB36" s="9">
         <f>IF(Y36=0,"",Z36/Y36)</f>
+        <v/>
+      </c>
+      <c r="AC36" s="8">
+        <f>D36+Y36</f>
+        <v/>
+      </c>
+      <c r="AD36" s="8">
+        <f>E36+Z36</f>
+        <v/>
+      </c>
+      <c r="AE36" s="8">
+        <f>AD36-AC36</f>
+        <v/>
+      </c>
+      <c r="AF36" s="9">
+        <f>IF(AC36=0,"",AD36/AC36)</f>
         <v/>
       </c>
     </row>
@@ -4124,11 +4652,11 @@
         <v/>
       </c>
       <c r="Y37" s="8">
-        <f>H37+L37+Q37+U37</f>
+        <f>L37+Q37+U37</f>
         <v/>
       </c>
       <c r="Z37" s="8">
-        <f>I37+N37+R37+V37</f>
+        <f>N37+R37+V37</f>
         <v/>
       </c>
       <c r="AA37" s="8">
@@ -4137,6 +4665,22 @@
       </c>
       <c r="AB37" s="9">
         <f>IF(Y37=0,"",Z37/Y37)</f>
+        <v/>
+      </c>
+      <c r="AC37" s="8">
+        <f>D37+Y37</f>
+        <v/>
+      </c>
+      <c r="AD37" s="8">
+        <f>E37+Z37</f>
+        <v/>
+      </c>
+      <c r="AE37" s="8">
+        <f>AD37-AC37</f>
+        <v/>
+      </c>
+      <c r="AF37" s="9">
+        <f>IF(AC37=0,"",AD37/AC37)</f>
         <v/>
       </c>
     </row>
@@ -4237,11 +4781,11 @@
         <v/>
       </c>
       <c r="Y38" s="5">
-        <f>H38+L38+Q38+U38</f>
+        <f>L38+Q38+U38</f>
         <v/>
       </c>
       <c r="Z38" s="5">
-        <f>I38+N38+R38+V38</f>
+        <f>N38+R38+V38</f>
         <v/>
       </c>
       <c r="AA38" s="5">
@@ -4250,6 +4794,22 @@
       </c>
       <c r="AB38" s="6">
         <f>IF(Y38=0,"",Z38/Y38)</f>
+        <v/>
+      </c>
+      <c r="AC38" s="5">
+        <f>D38+Y38</f>
+        <v/>
+      </c>
+      <c r="AD38" s="5">
+        <f>E38+Z38</f>
+        <v/>
+      </c>
+      <c r="AE38" s="5">
+        <f>AD38-AC38</f>
+        <v/>
+      </c>
+      <c r="AF38" s="6">
+        <f>IF(AC38=0,"",AD38/AC38)</f>
         <v/>
       </c>
     </row>
@@ -4343,11 +4903,11 @@
         <v/>
       </c>
       <c r="Y39" s="8">
-        <f>H39+L39+Q39+U39</f>
+        <f>L39+Q39+U39</f>
         <v/>
       </c>
       <c r="Z39" s="8">
-        <f>I39+N39+R39+V39</f>
+        <f>N39+R39+V39</f>
         <v/>
       </c>
       <c r="AA39" s="8">
@@ -4356,6 +4916,22 @@
       </c>
       <c r="AB39" s="9">
         <f>IF(Y39=0,"",Z39/Y39)</f>
+        <v/>
+      </c>
+      <c r="AC39" s="8">
+        <f>D39+Y39</f>
+        <v/>
+      </c>
+      <c r="AD39" s="8">
+        <f>E39+Z39</f>
+        <v/>
+      </c>
+      <c r="AE39" s="8">
+        <f>AD39-AC39</f>
+        <v/>
+      </c>
+      <c r="AF39" s="9">
+        <f>IF(AC39=0,"",AD39/AC39)</f>
         <v/>
       </c>
     </row>
@@ -4449,11 +5025,11 @@
         <v/>
       </c>
       <c r="Y40" s="8">
-        <f>H40+L40+Q40+U40</f>
+        <f>L40+Q40+U40</f>
         <v/>
       </c>
       <c r="Z40" s="8">
-        <f>I40+N40+R40+V40</f>
+        <f>N40+R40+V40</f>
         <v/>
       </c>
       <c r="AA40" s="8">
@@ -4462,6 +5038,22 @@
       </c>
       <c r="AB40" s="9">
         <f>IF(Y40=0,"",Z40/Y40)</f>
+        <v/>
+      </c>
+      <c r="AC40" s="8">
+        <f>D40+Y40</f>
+        <v/>
+      </c>
+      <c r="AD40" s="8">
+        <f>E40+Z40</f>
+        <v/>
+      </c>
+      <c r="AE40" s="8">
+        <f>AD40-AC40</f>
+        <v/>
+      </c>
+      <c r="AF40" s="9">
+        <f>IF(AC40=0,"",AD40/AC40)</f>
         <v/>
       </c>
     </row>
@@ -4555,11 +5147,11 @@
         <v/>
       </c>
       <c r="Y41" s="8">
-        <f>H41+L41+Q41+U41</f>
+        <f>L41+Q41+U41</f>
         <v/>
       </c>
       <c r="Z41" s="8">
-        <f>I41+N41+R41+V41</f>
+        <f>N41+R41+V41</f>
         <v/>
       </c>
       <c r="AA41" s="8">
@@ -4568,6 +5160,22 @@
       </c>
       <c r="AB41" s="9">
         <f>IF(Y41=0,"",Z41/Y41)</f>
+        <v/>
+      </c>
+      <c r="AC41" s="8">
+        <f>D41+Y41</f>
+        <v/>
+      </c>
+      <c r="AD41" s="8">
+        <f>E41+Z41</f>
+        <v/>
+      </c>
+      <c r="AE41" s="8">
+        <f>AD41-AC41</f>
+        <v/>
+      </c>
+      <c r="AF41" s="9">
+        <f>IF(AC41=0,"",AD41/AC41)</f>
         <v/>
       </c>
     </row>
@@ -4668,11 +5276,11 @@
         <v/>
       </c>
       <c r="Y42" s="5">
-        <f>H42+L42+Q42+U42</f>
+        <f>L42+Q42+U42</f>
         <v/>
       </c>
       <c r="Z42" s="5">
-        <f>I42+N42+R42+V42</f>
+        <f>N42+R42+V42</f>
         <v/>
       </c>
       <c r="AA42" s="5">
@@ -4681,6 +5289,22 @@
       </c>
       <c r="AB42" s="6">
         <f>IF(Y42=0,"",Z42/Y42)</f>
+        <v/>
+      </c>
+      <c r="AC42" s="5">
+        <f>D42+Y42</f>
+        <v/>
+      </c>
+      <c r="AD42" s="5">
+        <f>E42+Z42</f>
+        <v/>
+      </c>
+      <c r="AE42" s="5">
+        <f>AD42-AC42</f>
+        <v/>
+      </c>
+      <c r="AF42" s="6">
+        <f>IF(AC42=0,"",AD42/AC42)</f>
         <v/>
       </c>
     </row>
@@ -4774,11 +5398,11 @@
         <v/>
       </c>
       <c r="Y43" s="8">
-        <f>H43+L43+Q43+U43</f>
+        <f>L43+Q43+U43</f>
         <v/>
       </c>
       <c r="Z43" s="8">
-        <f>I43+N43+R43+V43</f>
+        <f>N43+R43+V43</f>
         <v/>
       </c>
       <c r="AA43" s="8">
@@ -4787,6 +5411,22 @@
       </c>
       <c r="AB43" s="9">
         <f>IF(Y43=0,"",Z43/Y43)</f>
+        <v/>
+      </c>
+      <c r="AC43" s="8">
+        <f>D43+Y43</f>
+        <v/>
+      </c>
+      <c r="AD43" s="8">
+        <f>E43+Z43</f>
+        <v/>
+      </c>
+      <c r="AE43" s="8">
+        <f>AD43-AC43</f>
+        <v/>
+      </c>
+      <c r="AF43" s="9">
+        <f>IF(AC43=0,"",AD43/AC43)</f>
         <v/>
       </c>
     </row>
@@ -4880,11 +5520,11 @@
         <v/>
       </c>
       <c r="Y44" s="8">
-        <f>H44+L44+Q44+U44</f>
+        <f>L44+Q44+U44</f>
         <v/>
       </c>
       <c r="Z44" s="8">
-        <f>I44+N44+R44+V44</f>
+        <f>N44+R44+V44</f>
         <v/>
       </c>
       <c r="AA44" s="8">
@@ -4893,6 +5533,22 @@
       </c>
       <c r="AB44" s="9">
         <f>IF(Y44=0,"",Z44/Y44)</f>
+        <v/>
+      </c>
+      <c r="AC44" s="8">
+        <f>D44+Y44</f>
+        <v/>
+      </c>
+      <c r="AD44" s="8">
+        <f>E44+Z44</f>
+        <v/>
+      </c>
+      <c r="AE44" s="8">
+        <f>AD44-AC44</f>
+        <v/>
+      </c>
+      <c r="AF44" s="9">
+        <f>IF(AC44=0,"",AD44/AC44)</f>
         <v/>
       </c>
     </row>
@@ -4986,11 +5642,11 @@
         <v/>
       </c>
       <c r="Y45" s="8">
-        <f>H45+L45+Q45+U45</f>
+        <f>L45+Q45+U45</f>
         <v/>
       </c>
       <c r="Z45" s="8">
-        <f>I45+N45+R45+V45</f>
+        <f>N45+R45+V45</f>
         <v/>
       </c>
       <c r="AA45" s="8">
@@ -4999,6 +5655,22 @@
       </c>
       <c r="AB45" s="9">
         <f>IF(Y45=0,"",Z45/Y45)</f>
+        <v/>
+      </c>
+      <c r="AC45" s="8">
+        <f>D45+Y45</f>
+        <v/>
+      </c>
+      <c r="AD45" s="8">
+        <f>E45+Z45</f>
+        <v/>
+      </c>
+      <c r="AE45" s="8">
+        <f>AD45-AC45</f>
+        <v/>
+      </c>
+      <c r="AF45" s="9">
+        <f>IF(AC45=0,"",AD45/AC45)</f>
         <v/>
       </c>
     </row>
@@ -5092,11 +5764,11 @@
         <v/>
       </c>
       <c r="Y46" s="8">
-        <f>H46+L46+Q46+U46</f>
+        <f>L46+Q46+U46</f>
         <v/>
       </c>
       <c r="Z46" s="8">
-        <f>I46+N46+R46+V46</f>
+        <f>N46+R46+V46</f>
         <v/>
       </c>
       <c r="AA46" s="8">
@@ -5105,6 +5777,22 @@
       </c>
       <c r="AB46" s="9">
         <f>IF(Y46=0,"",Z46/Y46)</f>
+        <v/>
+      </c>
+      <c r="AC46" s="8">
+        <f>D46+Y46</f>
+        <v/>
+      </c>
+      <c r="AD46" s="8">
+        <f>E46+Z46</f>
+        <v/>
+      </c>
+      <c r="AE46" s="8">
+        <f>AD46-AC46</f>
+        <v/>
+      </c>
+      <c r="AF46" s="9">
+        <f>IF(AC46=0,"",AD46/AC46)</f>
         <v/>
       </c>
     </row>
@@ -5205,11 +5893,11 @@
         <v/>
       </c>
       <c r="Y47" s="5">
-        <f>H47+L47+Q47+U47</f>
+        <f>L47+Q47+U47</f>
         <v/>
       </c>
       <c r="Z47" s="5">
-        <f>I47+N47+R47+V47</f>
+        <f>N47+R47+V47</f>
         <v/>
       </c>
       <c r="AA47" s="5">
@@ -5218,6 +5906,22 @@
       </c>
       <c r="AB47" s="6">
         <f>IF(Y47=0,"",Z47/Y47)</f>
+        <v/>
+      </c>
+      <c r="AC47" s="5">
+        <f>D47+Y47</f>
+        <v/>
+      </c>
+      <c r="AD47" s="5">
+        <f>E47+Z47</f>
+        <v/>
+      </c>
+      <c r="AE47" s="5">
+        <f>AD47-AC47</f>
+        <v/>
+      </c>
+      <c r="AF47" s="6">
+        <f>IF(AC47=0,"",AD47/AC47)</f>
         <v/>
       </c>
     </row>
@@ -5311,11 +6015,11 @@
         <v/>
       </c>
       <c r="Y48" s="8">
-        <f>H48+L48+Q48+U48</f>
+        <f>L48+Q48+U48</f>
         <v/>
       </c>
       <c r="Z48" s="8">
-        <f>I48+N48+R48+V48</f>
+        <f>N48+R48+V48</f>
         <v/>
       </c>
       <c r="AA48" s="8">
@@ -5324,6 +6028,22 @@
       </c>
       <c r="AB48" s="9">
         <f>IF(Y48=0,"",Z48/Y48)</f>
+        <v/>
+      </c>
+      <c r="AC48" s="8">
+        <f>D48+Y48</f>
+        <v/>
+      </c>
+      <c r="AD48" s="8">
+        <f>E48+Z48</f>
+        <v/>
+      </c>
+      <c r="AE48" s="8">
+        <f>AD48-AC48</f>
+        <v/>
+      </c>
+      <c r="AF48" s="9">
+        <f>IF(AC48=0,"",AD48/AC48)</f>
         <v/>
       </c>
     </row>
@@ -5420,11 +6140,11 @@
         <v/>
       </c>
       <c r="Y49" s="11">
-        <f>H49+L49+Q49+U49</f>
+        <f>L49+Q49+U49</f>
         <v/>
       </c>
       <c r="Z49" s="11">
-        <f>I49+N49+R49+V49</f>
+        <f>N49+R49+V49</f>
         <v/>
       </c>
       <c r="AA49" s="11">
@@ -5435,10 +6155,25 @@
         <f>IF(Y49=0,"",Z49/Y49)</f>
         <v/>
       </c>
+      <c r="AC49" s="11">
+        <f>D49+Y49</f>
+        <v/>
+      </c>
+      <c r="AD49" s="11">
+        <f>E49+Z49</f>
+        <v/>
+      </c>
+      <c r="AE49" s="11">
+        <f>AD49-AC49</f>
+        <v/>
+      </c>
+      <c r="AF49" s="12">
+        <f>IF(AC49=0,"",AD49/AC49)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A2:AB2"/>
+  <mergeCells count="11">
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="L4:P4"/>
     <mergeCell ref="B4:B5"/>
@@ -5447,6 +6182,8 @@
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="U4:X4"/>
     <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="AC4:AF4"/>
+    <mergeCell ref="A2:AF2"/>
     <mergeCell ref="D4:G4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5459,7 +6196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AF49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5490,6 +6227,10 @@
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5502,7 +6243,7 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأسوأ: لكل شهر، أدنى قيمة تاريخية لنفس الشهر (2023–2025) × معامل الاتجاه (بحد أقصى 1)، ولا يقل أكتوبر عن المحصل حتى تاريخه.</t>
+          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأسوأ: لكل شهر، أدنى قيمة تاريخية لنفس الشهر (2023–2025) × معامل الاتجاه (بحد أقصى 1)، ولا يقل أكتوبر عن المحصل حتى تاريخه.</t>
         </is>
       </c>
     </row>
@@ -5532,7 +6273,7 @@
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>سبتمبر (فعلي)</t>
+          <t>منها سبتمبر (مشمول في التراكمي، لا يُجمع معه)</t>
         </is>
       </c>
       <c r="I4" s="3" t="n"/>
@@ -5565,12 +6306,20 @@
       <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>المجموع سبتمبر–ديسمبر</t>
+          <t>المجموع أكتوبر–ديسمبر</t>
         </is>
       </c>
       <c r="Z4" s="3" t="n"/>
       <c r="AA4" s="3" t="n"/>
       <c r="AB4" s="3" t="n"/>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>إجمالي السنة 2026 (يناير–ديسمبر)</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="n"/>
+      <c r="AE4" s="3" t="n"/>
+      <c r="AF4" s="3" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="3" t="n"/>
@@ -5688,7 +6437,7 @@
       </c>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>المحصل + المتوقع</t>
+          <t>المتوقع</t>
         </is>
       </c>
       <c r="AA5" s="3" t="inlineStr">
@@ -5697,6 +6446,26 @@
         </is>
       </c>
       <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف السنوي</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل الفعلي + المتوقع</t>
+        </is>
+      </c>
+      <c r="AE5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="AF5" s="3" t="inlineStr">
         <is>
           <t>% من المستهدف</t>
         </is>
@@ -5799,11 +6568,11 @@
         <v/>
       </c>
       <c r="Y6" s="5">
-        <f>H6+L6+Q6+U6</f>
+        <f>L6+Q6+U6</f>
         <v/>
       </c>
       <c r="Z6" s="5">
-        <f>I6+N6+R6+V6</f>
+        <f>N6+R6+V6</f>
         <v/>
       </c>
       <c r="AA6" s="5">
@@ -5812,6 +6581,22 @@
       </c>
       <c r="AB6" s="6">
         <f>IF(Y6=0,"",Z6/Y6)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="5">
+        <f>D6+Y6</f>
+        <v/>
+      </c>
+      <c r="AD6" s="5">
+        <f>E6+Z6</f>
+        <v/>
+      </c>
+      <c r="AE6" s="5">
+        <f>AD6-AC6</f>
+        <v/>
+      </c>
+      <c r="AF6" s="6">
+        <f>IF(AC6=0,"",AD6/AC6)</f>
         <v/>
       </c>
     </row>
@@ -5905,11 +6690,11 @@
         <v/>
       </c>
       <c r="Y7" s="8">
-        <f>H7+L7+Q7+U7</f>
+        <f>L7+Q7+U7</f>
         <v/>
       </c>
       <c r="Z7" s="8">
-        <f>I7+N7+R7+V7</f>
+        <f>N7+R7+V7</f>
         <v/>
       </c>
       <c r="AA7" s="8">
@@ -5918,6 +6703,22 @@
       </c>
       <c r="AB7" s="9">
         <f>IF(Y7=0,"",Z7/Y7)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="8">
+        <f>D7+Y7</f>
+        <v/>
+      </c>
+      <c r="AD7" s="8">
+        <f>E7+Z7</f>
+        <v/>
+      </c>
+      <c r="AE7" s="8">
+        <f>AD7-AC7</f>
+        <v/>
+      </c>
+      <c r="AF7" s="9">
+        <f>IF(AC7=0,"",AD7/AC7)</f>
         <v/>
       </c>
     </row>
@@ -6011,11 +6812,11 @@
         <v/>
       </c>
       <c r="Y8" s="8">
-        <f>H8+L8+Q8+U8</f>
+        <f>L8+Q8+U8</f>
         <v/>
       </c>
       <c r="Z8" s="8">
-        <f>I8+N8+R8+V8</f>
+        <f>N8+R8+V8</f>
         <v/>
       </c>
       <c r="AA8" s="8">
@@ -6024,6 +6825,22 @@
       </c>
       <c r="AB8" s="9">
         <f>IF(Y8=0,"",Z8/Y8)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="8">
+        <f>D8+Y8</f>
+        <v/>
+      </c>
+      <c r="AD8" s="8">
+        <f>E8+Z8</f>
+        <v/>
+      </c>
+      <c r="AE8" s="8">
+        <f>AD8-AC8</f>
+        <v/>
+      </c>
+      <c r="AF8" s="9">
+        <f>IF(AC8=0,"",AD8/AC8)</f>
         <v/>
       </c>
     </row>
@@ -6117,11 +6934,11 @@
         <v/>
       </c>
       <c r="Y9" s="8">
-        <f>H9+L9+Q9+U9</f>
+        <f>L9+Q9+U9</f>
         <v/>
       </c>
       <c r="Z9" s="8">
-        <f>I9+N9+R9+V9</f>
+        <f>N9+R9+V9</f>
         <v/>
       </c>
       <c r="AA9" s="8">
@@ -6130,6 +6947,22 @@
       </c>
       <c r="AB9" s="9">
         <f>IF(Y9=0,"",Z9/Y9)</f>
+        <v/>
+      </c>
+      <c r="AC9" s="8">
+        <f>D9+Y9</f>
+        <v/>
+      </c>
+      <c r="AD9" s="8">
+        <f>E9+Z9</f>
+        <v/>
+      </c>
+      <c r="AE9" s="8">
+        <f>AD9-AC9</f>
+        <v/>
+      </c>
+      <c r="AF9" s="9">
+        <f>IF(AC9=0,"",AD9/AC9)</f>
         <v/>
       </c>
     </row>
@@ -6223,11 +7056,11 @@
         <v/>
       </c>
       <c r="Y10" s="8">
-        <f>H10+L10+Q10+U10</f>
+        <f>L10+Q10+U10</f>
         <v/>
       </c>
       <c r="Z10" s="8">
-        <f>I10+N10+R10+V10</f>
+        <f>N10+R10+V10</f>
         <v/>
       </c>
       <c r="AA10" s="8">
@@ -6236,6 +7069,22 @@
       </c>
       <c r="AB10" s="9">
         <f>IF(Y10=0,"",Z10/Y10)</f>
+        <v/>
+      </c>
+      <c r="AC10" s="8">
+        <f>D10+Y10</f>
+        <v/>
+      </c>
+      <c r="AD10" s="8">
+        <f>E10+Z10</f>
+        <v/>
+      </c>
+      <c r="AE10" s="8">
+        <f>AD10-AC10</f>
+        <v/>
+      </c>
+      <c r="AF10" s="9">
+        <f>IF(AC10=0,"",AD10/AC10)</f>
         <v/>
       </c>
     </row>
@@ -6329,11 +7178,11 @@
         <v/>
       </c>
       <c r="Y11" s="8">
-        <f>H11+L11+Q11+U11</f>
+        <f>L11+Q11+U11</f>
         <v/>
       </c>
       <c r="Z11" s="8">
-        <f>I11+N11+R11+V11</f>
+        <f>N11+R11+V11</f>
         <v/>
       </c>
       <c r="AA11" s="8">
@@ -6342,6 +7191,22 @@
       </c>
       <c r="AB11" s="9">
         <f>IF(Y11=0,"",Z11/Y11)</f>
+        <v/>
+      </c>
+      <c r="AC11" s="8">
+        <f>D11+Y11</f>
+        <v/>
+      </c>
+      <c r="AD11" s="8">
+        <f>E11+Z11</f>
+        <v/>
+      </c>
+      <c r="AE11" s="8">
+        <f>AD11-AC11</f>
+        <v/>
+      </c>
+      <c r="AF11" s="9">
+        <f>IF(AC11=0,"",AD11/AC11)</f>
         <v/>
       </c>
     </row>
@@ -6435,11 +7300,11 @@
         <v/>
       </c>
       <c r="Y12" s="8">
-        <f>H12+L12+Q12+U12</f>
+        <f>L12+Q12+U12</f>
         <v/>
       </c>
       <c r="Z12" s="8">
-        <f>I12+N12+R12+V12</f>
+        <f>N12+R12+V12</f>
         <v/>
       </c>
       <c r="AA12" s="8">
@@ -6448,6 +7313,22 @@
       </c>
       <c r="AB12" s="9">
         <f>IF(Y12=0,"",Z12/Y12)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="8">
+        <f>D12+Y12</f>
+        <v/>
+      </c>
+      <c r="AD12" s="8">
+        <f>E12+Z12</f>
+        <v/>
+      </c>
+      <c r="AE12" s="8">
+        <f>AD12-AC12</f>
+        <v/>
+      </c>
+      <c r="AF12" s="9">
+        <f>IF(AC12=0,"",AD12/AC12)</f>
         <v/>
       </c>
     </row>
@@ -6541,11 +7422,11 @@
         <v/>
       </c>
       <c r="Y13" s="8">
-        <f>H13+L13+Q13+U13</f>
+        <f>L13+Q13+U13</f>
         <v/>
       </c>
       <c r="Z13" s="8">
-        <f>I13+N13+R13+V13</f>
+        <f>N13+R13+V13</f>
         <v/>
       </c>
       <c r="AA13" s="8">
@@ -6554,6 +7435,22 @@
       </c>
       <c r="AB13" s="9">
         <f>IF(Y13=0,"",Z13/Y13)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="8">
+        <f>D13+Y13</f>
+        <v/>
+      </c>
+      <c r="AD13" s="8">
+        <f>E13+Z13</f>
+        <v/>
+      </c>
+      <c r="AE13" s="8">
+        <f>AD13-AC13</f>
+        <v/>
+      </c>
+      <c r="AF13" s="9">
+        <f>IF(AC13=0,"",AD13/AC13)</f>
         <v/>
       </c>
     </row>
@@ -6654,11 +7551,11 @@
         <v/>
       </c>
       <c r="Y14" s="5">
-        <f>H14+L14+Q14+U14</f>
+        <f>L14+Q14+U14</f>
         <v/>
       </c>
       <c r="Z14" s="5">
-        <f>I14+N14+R14+V14</f>
+        <f>N14+R14+V14</f>
         <v/>
       </c>
       <c r="AA14" s="5">
@@ -6667,6 +7564,22 @@
       </c>
       <c r="AB14" s="6">
         <f>IF(Y14=0,"",Z14/Y14)</f>
+        <v/>
+      </c>
+      <c r="AC14" s="5">
+        <f>D14+Y14</f>
+        <v/>
+      </c>
+      <c r="AD14" s="5">
+        <f>E14+Z14</f>
+        <v/>
+      </c>
+      <c r="AE14" s="5">
+        <f>AD14-AC14</f>
+        <v/>
+      </c>
+      <c r="AF14" s="6">
+        <f>IF(AC14=0,"",AD14/AC14)</f>
         <v/>
       </c>
     </row>
@@ -6760,11 +7673,11 @@
         <v/>
       </c>
       <c r="Y15" s="8">
-        <f>H15+L15+Q15+U15</f>
+        <f>L15+Q15+U15</f>
         <v/>
       </c>
       <c r="Z15" s="8">
-        <f>I15+N15+R15+V15</f>
+        <f>N15+R15+V15</f>
         <v/>
       </c>
       <c r="AA15" s="8">
@@ -6773,6 +7686,22 @@
       </c>
       <c r="AB15" s="9">
         <f>IF(Y15=0,"",Z15/Y15)</f>
+        <v/>
+      </c>
+      <c r="AC15" s="8">
+        <f>D15+Y15</f>
+        <v/>
+      </c>
+      <c r="AD15" s="8">
+        <f>E15+Z15</f>
+        <v/>
+      </c>
+      <c r="AE15" s="8">
+        <f>AD15-AC15</f>
+        <v/>
+      </c>
+      <c r="AF15" s="9">
+        <f>IF(AC15=0,"",AD15/AC15)</f>
         <v/>
       </c>
     </row>
@@ -6866,11 +7795,11 @@
         <v/>
       </c>
       <c r="Y16" s="8">
-        <f>H16+L16+Q16+U16</f>
+        <f>L16+Q16+U16</f>
         <v/>
       </c>
       <c r="Z16" s="8">
-        <f>I16+N16+R16+V16</f>
+        <f>N16+R16+V16</f>
         <v/>
       </c>
       <c r="AA16" s="8">
@@ -6879,6 +7808,22 @@
       </c>
       <c r="AB16" s="9">
         <f>IF(Y16=0,"",Z16/Y16)</f>
+        <v/>
+      </c>
+      <c r="AC16" s="8">
+        <f>D16+Y16</f>
+        <v/>
+      </c>
+      <c r="AD16" s="8">
+        <f>E16+Z16</f>
+        <v/>
+      </c>
+      <c r="AE16" s="8">
+        <f>AD16-AC16</f>
+        <v/>
+      </c>
+      <c r="AF16" s="9">
+        <f>IF(AC16=0,"",AD16/AC16)</f>
         <v/>
       </c>
     </row>
@@ -6972,11 +7917,11 @@
         <v/>
       </c>
       <c r="Y17" s="8">
-        <f>H17+L17+Q17+U17</f>
+        <f>L17+Q17+U17</f>
         <v/>
       </c>
       <c r="Z17" s="8">
-        <f>I17+N17+R17+V17</f>
+        <f>N17+R17+V17</f>
         <v/>
       </c>
       <c r="AA17" s="8">
@@ -6985,6 +7930,22 @@
       </c>
       <c r="AB17" s="9">
         <f>IF(Y17=0,"",Z17/Y17)</f>
+        <v/>
+      </c>
+      <c r="AC17" s="8">
+        <f>D17+Y17</f>
+        <v/>
+      </c>
+      <c r="AD17" s="8">
+        <f>E17+Z17</f>
+        <v/>
+      </c>
+      <c r="AE17" s="8">
+        <f>AD17-AC17</f>
+        <v/>
+      </c>
+      <c r="AF17" s="9">
+        <f>IF(AC17=0,"",AD17/AC17)</f>
         <v/>
       </c>
     </row>
@@ -7078,11 +8039,11 @@
         <v/>
       </c>
       <c r="Y18" s="8">
-        <f>H18+L18+Q18+U18</f>
+        <f>L18+Q18+U18</f>
         <v/>
       </c>
       <c r="Z18" s="8">
-        <f>I18+N18+R18+V18</f>
+        <f>N18+R18+V18</f>
         <v/>
       </c>
       <c r="AA18" s="8">
@@ -7091,6 +8052,22 @@
       </c>
       <c r="AB18" s="9">
         <f>IF(Y18=0,"",Z18/Y18)</f>
+        <v/>
+      </c>
+      <c r="AC18" s="8">
+        <f>D18+Y18</f>
+        <v/>
+      </c>
+      <c r="AD18" s="8">
+        <f>E18+Z18</f>
+        <v/>
+      </c>
+      <c r="AE18" s="8">
+        <f>AD18-AC18</f>
+        <v/>
+      </c>
+      <c r="AF18" s="9">
+        <f>IF(AC18=0,"",AD18/AC18)</f>
         <v/>
       </c>
     </row>
@@ -7184,11 +8161,11 @@
         <v/>
       </c>
       <c r="Y19" s="8">
-        <f>H19+L19+Q19+U19</f>
+        <f>L19+Q19+U19</f>
         <v/>
       </c>
       <c r="Z19" s="8">
-        <f>I19+N19+R19+V19</f>
+        <f>N19+R19+V19</f>
         <v/>
       </c>
       <c r="AA19" s="8">
@@ -7197,6 +8174,22 @@
       </c>
       <c r="AB19" s="9">
         <f>IF(Y19=0,"",Z19/Y19)</f>
+        <v/>
+      </c>
+      <c r="AC19" s="8">
+        <f>D19+Y19</f>
+        <v/>
+      </c>
+      <c r="AD19" s="8">
+        <f>E19+Z19</f>
+        <v/>
+      </c>
+      <c r="AE19" s="8">
+        <f>AD19-AC19</f>
+        <v/>
+      </c>
+      <c r="AF19" s="9">
+        <f>IF(AC19=0,"",AD19/AC19)</f>
         <v/>
       </c>
     </row>
@@ -7290,11 +8283,11 @@
         <v/>
       </c>
       <c r="Y20" s="8">
-        <f>H20+L20+Q20+U20</f>
+        <f>L20+Q20+U20</f>
         <v/>
       </c>
       <c r="Z20" s="8">
-        <f>I20+N20+R20+V20</f>
+        <f>N20+R20+V20</f>
         <v/>
       </c>
       <c r="AA20" s="8">
@@ -7303,6 +8296,22 @@
       </c>
       <c r="AB20" s="9">
         <f>IF(Y20=0,"",Z20/Y20)</f>
+        <v/>
+      </c>
+      <c r="AC20" s="8">
+        <f>D20+Y20</f>
+        <v/>
+      </c>
+      <c r="AD20" s="8">
+        <f>E20+Z20</f>
+        <v/>
+      </c>
+      <c r="AE20" s="8">
+        <f>AD20-AC20</f>
+        <v/>
+      </c>
+      <c r="AF20" s="9">
+        <f>IF(AC20=0,"",AD20/AC20)</f>
         <v/>
       </c>
     </row>
@@ -7396,11 +8405,11 @@
         <v/>
       </c>
       <c r="Y21" s="8">
-        <f>H21+L21+Q21+U21</f>
+        <f>L21+Q21+U21</f>
         <v/>
       </c>
       <c r="Z21" s="8">
-        <f>I21+N21+R21+V21</f>
+        <f>N21+R21+V21</f>
         <v/>
       </c>
       <c r="AA21" s="8">
@@ -7409,6 +8418,22 @@
       </c>
       <c r="AB21" s="9">
         <f>IF(Y21=0,"",Z21/Y21)</f>
+        <v/>
+      </c>
+      <c r="AC21" s="8">
+        <f>D21+Y21</f>
+        <v/>
+      </c>
+      <c r="AD21" s="8">
+        <f>E21+Z21</f>
+        <v/>
+      </c>
+      <c r="AE21" s="8">
+        <f>AD21-AC21</f>
+        <v/>
+      </c>
+      <c r="AF21" s="9">
+        <f>IF(AC21=0,"",AD21/AC21)</f>
         <v/>
       </c>
     </row>
@@ -7502,11 +8527,11 @@
         <v/>
       </c>
       <c r="Y22" s="8">
-        <f>H22+L22+Q22+U22</f>
+        <f>L22+Q22+U22</f>
         <v/>
       </c>
       <c r="Z22" s="8">
-        <f>I22+N22+R22+V22</f>
+        <f>N22+R22+V22</f>
         <v/>
       </c>
       <c r="AA22" s="8">
@@ -7515,6 +8540,22 @@
       </c>
       <c r="AB22" s="9">
         <f>IF(Y22=0,"",Z22/Y22)</f>
+        <v/>
+      </c>
+      <c r="AC22" s="8">
+        <f>D22+Y22</f>
+        <v/>
+      </c>
+      <c r="AD22" s="8">
+        <f>E22+Z22</f>
+        <v/>
+      </c>
+      <c r="AE22" s="8">
+        <f>AD22-AC22</f>
+        <v/>
+      </c>
+      <c r="AF22" s="9">
+        <f>IF(AC22=0,"",AD22/AC22)</f>
         <v/>
       </c>
     </row>
@@ -7608,11 +8649,11 @@
         <v/>
       </c>
       <c r="Y23" s="8">
-        <f>H23+L23+Q23+U23</f>
+        <f>L23+Q23+U23</f>
         <v/>
       </c>
       <c r="Z23" s="8">
-        <f>I23+N23+R23+V23</f>
+        <f>N23+R23+V23</f>
         <v/>
       </c>
       <c r="AA23" s="8">
@@ -7621,6 +8662,22 @@
       </c>
       <c r="AB23" s="9">
         <f>IF(Y23=0,"",Z23/Y23)</f>
+        <v/>
+      </c>
+      <c r="AC23" s="8">
+        <f>D23+Y23</f>
+        <v/>
+      </c>
+      <c r="AD23" s="8">
+        <f>E23+Z23</f>
+        <v/>
+      </c>
+      <c r="AE23" s="8">
+        <f>AD23-AC23</f>
+        <v/>
+      </c>
+      <c r="AF23" s="9">
+        <f>IF(AC23=0,"",AD23/AC23)</f>
         <v/>
       </c>
     </row>
@@ -7714,11 +8771,11 @@
         <v/>
       </c>
       <c r="Y24" s="8">
-        <f>H24+L24+Q24+U24</f>
+        <f>L24+Q24+U24</f>
         <v/>
       </c>
       <c r="Z24" s="8">
-        <f>I24+N24+R24+V24</f>
+        <f>N24+R24+V24</f>
         <v/>
       </c>
       <c r="AA24" s="8">
@@ -7727,6 +8784,22 @@
       </c>
       <c r="AB24" s="9">
         <f>IF(Y24=0,"",Z24/Y24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="8">
+        <f>D24+Y24</f>
+        <v/>
+      </c>
+      <c r="AD24" s="8">
+        <f>E24+Z24</f>
+        <v/>
+      </c>
+      <c r="AE24" s="8">
+        <f>AD24-AC24</f>
+        <v/>
+      </c>
+      <c r="AF24" s="9">
+        <f>IF(AC24=0,"",AD24/AC24)</f>
         <v/>
       </c>
     </row>
@@ -7820,11 +8893,11 @@
         <v/>
       </c>
       <c r="Y25" s="8">
-        <f>H25+L25+Q25+U25</f>
+        <f>L25+Q25+U25</f>
         <v/>
       </c>
       <c r="Z25" s="8">
-        <f>I25+N25+R25+V25</f>
+        <f>N25+R25+V25</f>
         <v/>
       </c>
       <c r="AA25" s="8">
@@ -7833,6 +8906,22 @@
       </c>
       <c r="AB25" s="9">
         <f>IF(Y25=0,"",Z25/Y25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="8">
+        <f>D25+Y25</f>
+        <v/>
+      </c>
+      <c r="AD25" s="8">
+        <f>E25+Z25</f>
+        <v/>
+      </c>
+      <c r="AE25" s="8">
+        <f>AD25-AC25</f>
+        <v/>
+      </c>
+      <c r="AF25" s="9">
+        <f>IF(AC25=0,"",AD25/AC25)</f>
         <v/>
       </c>
     </row>
@@ -7926,11 +9015,11 @@
         <v/>
       </c>
       <c r="Y26" s="8">
-        <f>H26+L26+Q26+U26</f>
+        <f>L26+Q26+U26</f>
         <v/>
       </c>
       <c r="Z26" s="8">
-        <f>I26+N26+R26+V26</f>
+        <f>N26+R26+V26</f>
         <v/>
       </c>
       <c r="AA26" s="8">
@@ -7939,6 +9028,22 @@
       </c>
       <c r="AB26" s="9">
         <f>IF(Y26=0,"",Z26/Y26)</f>
+        <v/>
+      </c>
+      <c r="AC26" s="8">
+        <f>D26+Y26</f>
+        <v/>
+      </c>
+      <c r="AD26" s="8">
+        <f>E26+Z26</f>
+        <v/>
+      </c>
+      <c r="AE26" s="8">
+        <f>AD26-AC26</f>
+        <v/>
+      </c>
+      <c r="AF26" s="9">
+        <f>IF(AC26=0,"",AD26/AC26)</f>
         <v/>
       </c>
     </row>
@@ -8032,11 +9137,11 @@
         <v/>
       </c>
       <c r="Y27" s="8">
-        <f>H27+L27+Q27+U27</f>
+        <f>L27+Q27+U27</f>
         <v/>
       </c>
       <c r="Z27" s="8">
-        <f>I27+N27+R27+V27</f>
+        <f>N27+R27+V27</f>
         <v/>
       </c>
       <c r="AA27" s="8">
@@ -8045,6 +9150,22 @@
       </c>
       <c r="AB27" s="9">
         <f>IF(Y27=0,"",Z27/Y27)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="8">
+        <f>D27+Y27</f>
+        <v/>
+      </c>
+      <c r="AD27" s="8">
+        <f>E27+Z27</f>
+        <v/>
+      </c>
+      <c r="AE27" s="8">
+        <f>AD27-AC27</f>
+        <v/>
+      </c>
+      <c r="AF27" s="9">
+        <f>IF(AC27=0,"",AD27/AC27)</f>
         <v/>
       </c>
     </row>
@@ -8138,11 +9259,11 @@
         <v/>
       </c>
       <c r="Y28" s="8">
-        <f>H28+L28+Q28+U28</f>
+        <f>L28+Q28+U28</f>
         <v/>
       </c>
       <c r="Z28" s="8">
-        <f>I28+N28+R28+V28</f>
+        <f>N28+R28+V28</f>
         <v/>
       </c>
       <c r="AA28" s="8">
@@ -8151,6 +9272,22 @@
       </c>
       <c r="AB28" s="9">
         <f>IF(Y28=0,"",Z28/Y28)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="8">
+        <f>D28+Y28</f>
+        <v/>
+      </c>
+      <c r="AD28" s="8">
+        <f>E28+Z28</f>
+        <v/>
+      </c>
+      <c r="AE28" s="8">
+        <f>AD28-AC28</f>
+        <v/>
+      </c>
+      <c r="AF28" s="9">
+        <f>IF(AC28=0,"",AD28/AC28)</f>
         <v/>
       </c>
     </row>
@@ -8244,11 +9381,11 @@
         <v/>
       </c>
       <c r="Y29" s="8">
-        <f>H29+L29+Q29+U29</f>
+        <f>L29+Q29+U29</f>
         <v/>
       </c>
       <c r="Z29" s="8">
-        <f>I29+N29+R29+V29</f>
+        <f>N29+R29+V29</f>
         <v/>
       </c>
       <c r="AA29" s="8">
@@ -8257,6 +9394,22 @@
       </c>
       <c r="AB29" s="9">
         <f>IF(Y29=0,"",Z29/Y29)</f>
+        <v/>
+      </c>
+      <c r="AC29" s="8">
+        <f>D29+Y29</f>
+        <v/>
+      </c>
+      <c r="AD29" s="8">
+        <f>E29+Z29</f>
+        <v/>
+      </c>
+      <c r="AE29" s="8">
+        <f>AD29-AC29</f>
+        <v/>
+      </c>
+      <c r="AF29" s="9">
+        <f>IF(AC29=0,"",AD29/AC29)</f>
         <v/>
       </c>
     </row>
@@ -8350,11 +9503,11 @@
         <v/>
       </c>
       <c r="Y30" s="8">
-        <f>H30+L30+Q30+U30</f>
+        <f>L30+Q30+U30</f>
         <v/>
       </c>
       <c r="Z30" s="8">
-        <f>I30+N30+R30+V30</f>
+        <f>N30+R30+V30</f>
         <v/>
       </c>
       <c r="AA30" s="8">
@@ -8363,6 +9516,22 @@
       </c>
       <c r="AB30" s="9">
         <f>IF(Y30=0,"",Z30/Y30)</f>
+        <v/>
+      </c>
+      <c r="AC30" s="8">
+        <f>D30+Y30</f>
+        <v/>
+      </c>
+      <c r="AD30" s="8">
+        <f>E30+Z30</f>
+        <v/>
+      </c>
+      <c r="AE30" s="8">
+        <f>AD30-AC30</f>
+        <v/>
+      </c>
+      <c r="AF30" s="9">
+        <f>IF(AC30=0,"",AD30/AC30)</f>
         <v/>
       </c>
     </row>
@@ -8456,11 +9625,11 @@
         <v/>
       </c>
       <c r="Y31" s="8">
-        <f>H31+L31+Q31+U31</f>
+        <f>L31+Q31+U31</f>
         <v/>
       </c>
       <c r="Z31" s="8">
-        <f>I31+N31+R31+V31</f>
+        <f>N31+R31+V31</f>
         <v/>
       </c>
       <c r="AA31" s="8">
@@ -8469,6 +9638,22 @@
       </c>
       <c r="AB31" s="9">
         <f>IF(Y31=0,"",Z31/Y31)</f>
+        <v/>
+      </c>
+      <c r="AC31" s="8">
+        <f>D31+Y31</f>
+        <v/>
+      </c>
+      <c r="AD31" s="8">
+        <f>E31+Z31</f>
+        <v/>
+      </c>
+      <c r="AE31" s="8">
+        <f>AD31-AC31</f>
+        <v/>
+      </c>
+      <c r="AF31" s="9">
+        <f>IF(AC31=0,"",AD31/AC31)</f>
         <v/>
       </c>
     </row>
@@ -8562,11 +9747,11 @@
         <v/>
       </c>
       <c r="Y32" s="8">
-        <f>H32+L32+Q32+U32</f>
+        <f>L32+Q32+U32</f>
         <v/>
       </c>
       <c r="Z32" s="8">
-        <f>I32+N32+R32+V32</f>
+        <f>N32+R32+V32</f>
         <v/>
       </c>
       <c r="AA32" s="8">
@@ -8575,6 +9760,22 @@
       </c>
       <c r="AB32" s="9">
         <f>IF(Y32=0,"",Z32/Y32)</f>
+        <v/>
+      </c>
+      <c r="AC32" s="8">
+        <f>D32+Y32</f>
+        <v/>
+      </c>
+      <c r="AD32" s="8">
+        <f>E32+Z32</f>
+        <v/>
+      </c>
+      <c r="AE32" s="8">
+        <f>AD32-AC32</f>
+        <v/>
+      </c>
+      <c r="AF32" s="9">
+        <f>IF(AC32=0,"",AD32/AC32)</f>
         <v/>
       </c>
     </row>
@@ -8675,11 +9876,11 @@
         <v/>
       </c>
       <c r="Y33" s="5">
-        <f>H33+L33+Q33+U33</f>
+        <f>L33+Q33+U33</f>
         <v/>
       </c>
       <c r="Z33" s="5">
-        <f>I33+N33+R33+V33</f>
+        <f>N33+R33+V33</f>
         <v/>
       </c>
       <c r="AA33" s="5">
@@ -8688,6 +9889,22 @@
       </c>
       <c r="AB33" s="6">
         <f>IF(Y33=0,"",Z33/Y33)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="5">
+        <f>D33+Y33</f>
+        <v/>
+      </c>
+      <c r="AD33" s="5">
+        <f>E33+Z33</f>
+        <v/>
+      </c>
+      <c r="AE33" s="5">
+        <f>AD33-AC33</f>
+        <v/>
+      </c>
+      <c r="AF33" s="6">
+        <f>IF(AC33=0,"",AD33/AC33)</f>
         <v/>
       </c>
     </row>
@@ -8781,11 +9998,11 @@
         <v/>
       </c>
       <c r="Y34" s="8">
-        <f>H34+L34+Q34+U34</f>
+        <f>L34+Q34+U34</f>
         <v/>
       </c>
       <c r="Z34" s="8">
-        <f>I34+N34+R34+V34</f>
+        <f>N34+R34+V34</f>
         <v/>
       </c>
       <c r="AA34" s="8">
@@ -8794,6 +10011,22 @@
       </c>
       <c r="AB34" s="9">
         <f>IF(Y34=0,"",Z34/Y34)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="8">
+        <f>D34+Y34</f>
+        <v/>
+      </c>
+      <c r="AD34" s="8">
+        <f>E34+Z34</f>
+        <v/>
+      </c>
+      <c r="AE34" s="8">
+        <f>AD34-AC34</f>
+        <v/>
+      </c>
+      <c r="AF34" s="9">
+        <f>IF(AC34=0,"",AD34/AC34)</f>
         <v/>
       </c>
     </row>
@@ -8887,11 +10120,11 @@
         <v/>
       </c>
       <c r="Y35" s="8">
-        <f>H35+L35+Q35+U35</f>
+        <f>L35+Q35+U35</f>
         <v/>
       </c>
       <c r="Z35" s="8">
-        <f>I35+N35+R35+V35</f>
+        <f>N35+R35+V35</f>
         <v/>
       </c>
       <c r="AA35" s="8">
@@ -8900,6 +10133,22 @@
       </c>
       <c r="AB35" s="9">
         <f>IF(Y35=0,"",Z35/Y35)</f>
+        <v/>
+      </c>
+      <c r="AC35" s="8">
+        <f>D35+Y35</f>
+        <v/>
+      </c>
+      <c r="AD35" s="8">
+        <f>E35+Z35</f>
+        <v/>
+      </c>
+      <c r="AE35" s="8">
+        <f>AD35-AC35</f>
+        <v/>
+      </c>
+      <c r="AF35" s="9">
+        <f>IF(AC35=0,"",AD35/AC35)</f>
         <v/>
       </c>
     </row>
@@ -8993,11 +10242,11 @@
         <v/>
       </c>
       <c r="Y36" s="8">
-        <f>H36+L36+Q36+U36</f>
+        <f>L36+Q36+U36</f>
         <v/>
       </c>
       <c r="Z36" s="8">
-        <f>I36+N36+R36+V36</f>
+        <f>N36+R36+V36</f>
         <v/>
       </c>
       <c r="AA36" s="8">
@@ -9006,6 +10255,22 @@
       </c>
       <c r="AB36" s="9">
         <f>IF(Y36=0,"",Z36/Y36)</f>
+        <v/>
+      </c>
+      <c r="AC36" s="8">
+        <f>D36+Y36</f>
+        <v/>
+      </c>
+      <c r="AD36" s="8">
+        <f>E36+Z36</f>
+        <v/>
+      </c>
+      <c r="AE36" s="8">
+        <f>AD36-AC36</f>
+        <v/>
+      </c>
+      <c r="AF36" s="9">
+        <f>IF(AC36=0,"",AD36/AC36)</f>
         <v/>
       </c>
     </row>
@@ -9099,11 +10364,11 @@
         <v/>
       </c>
       <c r="Y37" s="8">
-        <f>H37+L37+Q37+U37</f>
+        <f>L37+Q37+U37</f>
         <v/>
       </c>
       <c r="Z37" s="8">
-        <f>I37+N37+R37+V37</f>
+        <f>N37+R37+V37</f>
         <v/>
       </c>
       <c r="AA37" s="8">
@@ -9112,6 +10377,22 @@
       </c>
       <c r="AB37" s="9">
         <f>IF(Y37=0,"",Z37/Y37)</f>
+        <v/>
+      </c>
+      <c r="AC37" s="8">
+        <f>D37+Y37</f>
+        <v/>
+      </c>
+      <c r="AD37" s="8">
+        <f>E37+Z37</f>
+        <v/>
+      </c>
+      <c r="AE37" s="8">
+        <f>AD37-AC37</f>
+        <v/>
+      </c>
+      <c r="AF37" s="9">
+        <f>IF(AC37=0,"",AD37/AC37)</f>
         <v/>
       </c>
     </row>
@@ -9212,11 +10493,11 @@
         <v/>
       </c>
       <c r="Y38" s="5">
-        <f>H38+L38+Q38+U38</f>
+        <f>L38+Q38+U38</f>
         <v/>
       </c>
       <c r="Z38" s="5">
-        <f>I38+N38+R38+V38</f>
+        <f>N38+R38+V38</f>
         <v/>
       </c>
       <c r="AA38" s="5">
@@ -9225,6 +10506,22 @@
       </c>
       <c r="AB38" s="6">
         <f>IF(Y38=0,"",Z38/Y38)</f>
+        <v/>
+      </c>
+      <c r="AC38" s="5">
+        <f>D38+Y38</f>
+        <v/>
+      </c>
+      <c r="AD38" s="5">
+        <f>E38+Z38</f>
+        <v/>
+      </c>
+      <c r="AE38" s="5">
+        <f>AD38-AC38</f>
+        <v/>
+      </c>
+      <c r="AF38" s="6">
+        <f>IF(AC38=0,"",AD38/AC38)</f>
         <v/>
       </c>
     </row>
@@ -9318,11 +10615,11 @@
         <v/>
       </c>
       <c r="Y39" s="8">
-        <f>H39+L39+Q39+U39</f>
+        <f>L39+Q39+U39</f>
         <v/>
       </c>
       <c r="Z39" s="8">
-        <f>I39+N39+R39+V39</f>
+        <f>N39+R39+V39</f>
         <v/>
       </c>
       <c r="AA39" s="8">
@@ -9331,6 +10628,22 @@
       </c>
       <c r="AB39" s="9">
         <f>IF(Y39=0,"",Z39/Y39)</f>
+        <v/>
+      </c>
+      <c r="AC39" s="8">
+        <f>D39+Y39</f>
+        <v/>
+      </c>
+      <c r="AD39" s="8">
+        <f>E39+Z39</f>
+        <v/>
+      </c>
+      <c r="AE39" s="8">
+        <f>AD39-AC39</f>
+        <v/>
+      </c>
+      <c r="AF39" s="9">
+        <f>IF(AC39=0,"",AD39/AC39)</f>
         <v/>
       </c>
     </row>
@@ -9424,11 +10737,11 @@
         <v/>
       </c>
       <c r="Y40" s="8">
-        <f>H40+L40+Q40+U40</f>
+        <f>L40+Q40+U40</f>
         <v/>
       </c>
       <c r="Z40" s="8">
-        <f>I40+N40+R40+V40</f>
+        <f>N40+R40+V40</f>
         <v/>
       </c>
       <c r="AA40" s="8">
@@ -9437,6 +10750,22 @@
       </c>
       <c r="AB40" s="9">
         <f>IF(Y40=0,"",Z40/Y40)</f>
+        <v/>
+      </c>
+      <c r="AC40" s="8">
+        <f>D40+Y40</f>
+        <v/>
+      </c>
+      <c r="AD40" s="8">
+        <f>E40+Z40</f>
+        <v/>
+      </c>
+      <c r="AE40" s="8">
+        <f>AD40-AC40</f>
+        <v/>
+      </c>
+      <c r="AF40" s="9">
+        <f>IF(AC40=0,"",AD40/AC40)</f>
         <v/>
       </c>
     </row>
@@ -9530,11 +10859,11 @@
         <v/>
       </c>
       <c r="Y41" s="8">
-        <f>H41+L41+Q41+U41</f>
+        <f>L41+Q41+U41</f>
         <v/>
       </c>
       <c r="Z41" s="8">
-        <f>I41+N41+R41+V41</f>
+        <f>N41+R41+V41</f>
         <v/>
       </c>
       <c r="AA41" s="8">
@@ -9543,6 +10872,22 @@
       </c>
       <c r="AB41" s="9">
         <f>IF(Y41=0,"",Z41/Y41)</f>
+        <v/>
+      </c>
+      <c r="AC41" s="8">
+        <f>D41+Y41</f>
+        <v/>
+      </c>
+      <c r="AD41" s="8">
+        <f>E41+Z41</f>
+        <v/>
+      </c>
+      <c r="AE41" s="8">
+        <f>AD41-AC41</f>
+        <v/>
+      </c>
+      <c r="AF41" s="9">
+        <f>IF(AC41=0,"",AD41/AC41)</f>
         <v/>
       </c>
     </row>
@@ -9643,11 +10988,11 @@
         <v/>
       </c>
       <c r="Y42" s="5">
-        <f>H42+L42+Q42+U42</f>
+        <f>L42+Q42+U42</f>
         <v/>
       </c>
       <c r="Z42" s="5">
-        <f>I42+N42+R42+V42</f>
+        <f>N42+R42+V42</f>
         <v/>
       </c>
       <c r="AA42" s="5">
@@ -9656,6 +11001,22 @@
       </c>
       <c r="AB42" s="6">
         <f>IF(Y42=0,"",Z42/Y42)</f>
+        <v/>
+      </c>
+      <c r="AC42" s="5">
+        <f>D42+Y42</f>
+        <v/>
+      </c>
+      <c r="AD42" s="5">
+        <f>E42+Z42</f>
+        <v/>
+      </c>
+      <c r="AE42" s="5">
+        <f>AD42-AC42</f>
+        <v/>
+      </c>
+      <c r="AF42" s="6">
+        <f>IF(AC42=0,"",AD42/AC42)</f>
         <v/>
       </c>
     </row>
@@ -9749,11 +11110,11 @@
         <v/>
       </c>
       <c r="Y43" s="8">
-        <f>H43+L43+Q43+U43</f>
+        <f>L43+Q43+U43</f>
         <v/>
       </c>
       <c r="Z43" s="8">
-        <f>I43+N43+R43+V43</f>
+        <f>N43+R43+V43</f>
         <v/>
       </c>
       <c r="AA43" s="8">
@@ -9762,6 +11123,22 @@
       </c>
       <c r="AB43" s="9">
         <f>IF(Y43=0,"",Z43/Y43)</f>
+        <v/>
+      </c>
+      <c r="AC43" s="8">
+        <f>D43+Y43</f>
+        <v/>
+      </c>
+      <c r="AD43" s="8">
+        <f>E43+Z43</f>
+        <v/>
+      </c>
+      <c r="AE43" s="8">
+        <f>AD43-AC43</f>
+        <v/>
+      </c>
+      <c r="AF43" s="9">
+        <f>IF(AC43=0,"",AD43/AC43)</f>
         <v/>
       </c>
     </row>
@@ -9855,11 +11232,11 @@
         <v/>
       </c>
       <c r="Y44" s="8">
-        <f>H44+L44+Q44+U44</f>
+        <f>L44+Q44+U44</f>
         <v/>
       </c>
       <c r="Z44" s="8">
-        <f>I44+N44+R44+V44</f>
+        <f>N44+R44+V44</f>
         <v/>
       </c>
       <c r="AA44" s="8">
@@ -9868,6 +11245,22 @@
       </c>
       <c r="AB44" s="9">
         <f>IF(Y44=0,"",Z44/Y44)</f>
+        <v/>
+      </c>
+      <c r="AC44" s="8">
+        <f>D44+Y44</f>
+        <v/>
+      </c>
+      <c r="AD44" s="8">
+        <f>E44+Z44</f>
+        <v/>
+      </c>
+      <c r="AE44" s="8">
+        <f>AD44-AC44</f>
+        <v/>
+      </c>
+      <c r="AF44" s="9">
+        <f>IF(AC44=0,"",AD44/AC44)</f>
         <v/>
       </c>
     </row>
@@ -9961,11 +11354,11 @@
         <v/>
       </c>
       <c r="Y45" s="8">
-        <f>H45+L45+Q45+U45</f>
+        <f>L45+Q45+U45</f>
         <v/>
       </c>
       <c r="Z45" s="8">
-        <f>I45+N45+R45+V45</f>
+        <f>N45+R45+V45</f>
         <v/>
       </c>
       <c r="AA45" s="8">
@@ -9974,6 +11367,22 @@
       </c>
       <c r="AB45" s="9">
         <f>IF(Y45=0,"",Z45/Y45)</f>
+        <v/>
+      </c>
+      <c r="AC45" s="8">
+        <f>D45+Y45</f>
+        <v/>
+      </c>
+      <c r="AD45" s="8">
+        <f>E45+Z45</f>
+        <v/>
+      </c>
+      <c r="AE45" s="8">
+        <f>AD45-AC45</f>
+        <v/>
+      </c>
+      <c r="AF45" s="9">
+        <f>IF(AC45=0,"",AD45/AC45)</f>
         <v/>
       </c>
     </row>
@@ -10067,11 +11476,11 @@
         <v/>
       </c>
       <c r="Y46" s="8">
-        <f>H46+L46+Q46+U46</f>
+        <f>L46+Q46+U46</f>
         <v/>
       </c>
       <c r="Z46" s="8">
-        <f>I46+N46+R46+V46</f>
+        <f>N46+R46+V46</f>
         <v/>
       </c>
       <c r="AA46" s="8">
@@ -10080,6 +11489,22 @@
       </c>
       <c r="AB46" s="9">
         <f>IF(Y46=0,"",Z46/Y46)</f>
+        <v/>
+      </c>
+      <c r="AC46" s="8">
+        <f>D46+Y46</f>
+        <v/>
+      </c>
+      <c r="AD46" s="8">
+        <f>E46+Z46</f>
+        <v/>
+      </c>
+      <c r="AE46" s="8">
+        <f>AD46-AC46</f>
+        <v/>
+      </c>
+      <c r="AF46" s="9">
+        <f>IF(AC46=0,"",AD46/AC46)</f>
         <v/>
       </c>
     </row>
@@ -10180,11 +11605,11 @@
         <v/>
       </c>
       <c r="Y47" s="5">
-        <f>H47+L47+Q47+U47</f>
+        <f>L47+Q47+U47</f>
         <v/>
       </c>
       <c r="Z47" s="5">
-        <f>I47+N47+R47+V47</f>
+        <f>N47+R47+V47</f>
         <v/>
       </c>
       <c r="AA47" s="5">
@@ -10193,6 +11618,22 @@
       </c>
       <c r="AB47" s="6">
         <f>IF(Y47=0,"",Z47/Y47)</f>
+        <v/>
+      </c>
+      <c r="AC47" s="5">
+        <f>D47+Y47</f>
+        <v/>
+      </c>
+      <c r="AD47" s="5">
+        <f>E47+Z47</f>
+        <v/>
+      </c>
+      <c r="AE47" s="5">
+        <f>AD47-AC47</f>
+        <v/>
+      </c>
+      <c r="AF47" s="6">
+        <f>IF(AC47=0,"",AD47/AC47)</f>
         <v/>
       </c>
     </row>
@@ -10286,11 +11727,11 @@
         <v/>
       </c>
       <c r="Y48" s="8">
-        <f>H48+L48+Q48+U48</f>
+        <f>L48+Q48+U48</f>
         <v/>
       </c>
       <c r="Z48" s="8">
-        <f>I48+N48+R48+V48</f>
+        <f>N48+R48+V48</f>
         <v/>
       </c>
       <c r="AA48" s="8">
@@ -10299,6 +11740,22 @@
       </c>
       <c r="AB48" s="9">
         <f>IF(Y48=0,"",Z48/Y48)</f>
+        <v/>
+      </c>
+      <c r="AC48" s="8">
+        <f>D48+Y48</f>
+        <v/>
+      </c>
+      <c r="AD48" s="8">
+        <f>E48+Z48</f>
+        <v/>
+      </c>
+      <c r="AE48" s="8">
+        <f>AD48-AC48</f>
+        <v/>
+      </c>
+      <c r="AF48" s="9">
+        <f>IF(AC48=0,"",AD48/AC48)</f>
         <v/>
       </c>
     </row>
@@ -10395,11 +11852,11 @@
         <v/>
       </c>
       <c r="Y49" s="11">
-        <f>H49+L49+Q49+U49</f>
+        <f>L49+Q49+U49</f>
         <v/>
       </c>
       <c r="Z49" s="11">
-        <f>I49+N49+R49+V49</f>
+        <f>N49+R49+V49</f>
         <v/>
       </c>
       <c r="AA49" s="11">
@@ -10410,10 +11867,25 @@
         <f>IF(Y49=0,"",Z49/Y49)</f>
         <v/>
       </c>
+      <c r="AC49" s="11">
+        <f>D49+Y49</f>
+        <v/>
+      </c>
+      <c r="AD49" s="11">
+        <f>E49+Z49</f>
+        <v/>
+      </c>
+      <c r="AE49" s="11">
+        <f>AD49-AC49</f>
+        <v/>
+      </c>
+      <c r="AF49" s="12">
+        <f>IF(AC49=0,"",AD49/AC49)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A2:AB2"/>
+  <mergeCells count="11">
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="L4:P4"/>
     <mergeCell ref="B4:B5"/>
@@ -10422,6 +11894,8 @@
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="U4:X4"/>
     <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="AC4:AF4"/>
+    <mergeCell ref="A2:AF2"/>
     <mergeCell ref="D4:G4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rebuild best/worst monthly workbook from user's edited closings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/المستهدف_الشهري_أفضل_أسوأ.xlsx
+++ b/المستهدف_الشهري_أفضل_أسوأ.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF49"/>
+  <dimension ref="A1:AF47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -524,14 +524,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل التراكمي حتى سبتمبر والشهري سبتمبر–ديسمبر 2026 — الأفضل (متفائل)</t>
+          <t>المستهدف والمحصل التراكمي حتى سبتمبر والشهري سبتمبر–ديسمبر 2026 — الأفضل (أرقامك المعدّلة)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأفضل: لكل شهر، الأكبر بين التوقع الأساسي ومتوسط أعلى قيمتين تاريخيتين لنفس الشهر (2023–2025) × معامل الاتجاه (لا يقل عن 1)، بسقف 1.5 ضعف الأساسي.</t>
+          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. الأفضل = عمود "إقفال 2026 – أساسي" في ملفك المعدّل لكل حساب. للحسابات التي عدّلتها وُزّع الباقي حتى نهاية السنة (إقفالك − الفعلي حتى تاريخه) على بقية أكتوبر ونوفمبر وديسمبر بنسب المستهدف الشهري للحساب؛ وغيرها بقي على توزيع التوقع الأساسي بالموسمية. لا ينزل أي حساب عن المحصل الفعلي.</t>
         </is>
       </c>
     </row>
@@ -896,19 +896,19 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>14155</t>
+          <t>142162</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ريع الأراضي (تأجير الأراض )</t>
+          <t>إيرادات  تأجير المرافق</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>428594563.82</v>
+        <v>539363594.54</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>612328416.96</v>
+        <v>428392037.77</v>
       </c>
       <c r="F7" s="8">
         <f>E7-D7</f>
@@ -919,10 +919,10 @@
         <v/>
       </c>
       <c r="H7" s="8" t="n">
-        <v>51408989.3</v>
+        <v>24198982.49</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>55595082.92</v>
+        <v>1895695.14</v>
       </c>
       <c r="J7" s="8">
         <f>I7-H7</f>
@@ -933,13 +933,13 @@
         <v/>
       </c>
       <c r="L7" s="8" t="n">
-        <v>199630948.23</v>
+        <v>28067945.58</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>32158747.69</v>
+        <v>322955.69</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>183778939.76</v>
+        <v>29528868.84</v>
       </c>
       <c r="O7" s="8">
         <f>N7-L7</f>
@@ -950,10 +950,10 @@
         <v/>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>66228430.48</v>
+        <v>418948643.78</v>
       </c>
       <c r="R7" s="8" t="n">
-        <v>136900856.43</v>
+        <v>441008548.03</v>
       </c>
       <c r="S7" s="8">
         <f>R7-Q7</f>
@@ -964,10 +964,10 @@
         <v/>
       </c>
       <c r="U7" s="8" t="n">
-        <v>42439465.39</v>
+        <v>16895879.24</v>
       </c>
       <c r="V7" s="8" t="n">
-        <v>79276888.41</v>
+        <v>17785538.35</v>
       </c>
       <c r="W7" s="8">
         <f>V7-U7</f>
@@ -1018,19 +1018,19 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>142162</t>
+          <t>14155</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>إيرادات  تأجير المرافق</t>
+          <t>ريع الأراضي (تأجير الأراض )</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>539363594.54</v>
+        <v>428594563.82</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>428392037.77</v>
+        <v>612328416.96</v>
       </c>
       <c r="F8" s="8">
         <f>E8-D8</f>
@@ -1041,10 +1041,10 @@
         <v/>
       </c>
       <c r="H8" s="8" t="n">
-        <v>24198982.49</v>
+        <v>51408989.3</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>1895695.14</v>
+        <v>55595082.92</v>
       </c>
       <c r="J8" s="8">
         <f>I8-H8</f>
@@ -1055,13 +1055,13 @@
         <v/>
       </c>
       <c r="L8" s="8" t="n">
-        <v>28067945.58</v>
+        <v>199630948.23</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>322955.69</v>
+        <v>32158747.69</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>984439.64</v>
+        <v>111711994.47</v>
       </c>
       <c r="O8" s="8">
         <f>N8-L8</f>
@@ -1072,10 +1072,10 @@
         <v/>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>418948643.78</v>
+        <v>66228430.48</v>
       </c>
       <c r="R8" s="8" t="n">
-        <v>33060558.07</v>
+        <v>31460067.15</v>
       </c>
       <c r="S8" s="8">
         <f>R8-Q8</f>
@@ -1086,10 +1086,10 @@
         <v/>
       </c>
       <c r="U8" s="8" t="n">
-        <v>16895879.24</v>
+        <v>42439465.39</v>
       </c>
       <c r="V8" s="8" t="n">
-        <v>26061705.75</v>
+        <v>20159747.42</v>
       </c>
       <c r="W8" s="8">
         <f>V8-U8</f>
@@ -1183,7 +1183,7 @@
         <v>380080</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>1745875.88</v>
+        <v>1438875</v>
       </c>
       <c r="O9" s="8">
         <f>N9-L9</f>
@@ -1197,7 +1197,7 @@
         <v>10001631.64</v>
       </c>
       <c r="R9" s="8" t="n">
-        <v>1445059.5</v>
+        <v>1393808.8</v>
       </c>
       <c r="S9" s="8">
         <f>R9-Q9</f>
@@ -1211,7 +1211,7 @@
         <v>3599329.08</v>
       </c>
       <c r="V9" s="8" t="n">
-        <v>687274.05</v>
+        <v>458182.7</v>
       </c>
       <c r="W9" s="8">
         <f>V9-U9</f>
@@ -1319,7 +1319,7 @@
         <v>150620.18</v>
       </c>
       <c r="R10" s="8" t="n">
-        <v>211919.02</v>
+        <v>194277.38</v>
       </c>
       <c r="S10" s="8">
         <f>R10-Q10</f>
@@ -1333,7 +1333,7 @@
         <v>150849.35</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>117531.54</v>
+        <v>78354.36</v>
       </c>
       <c r="W10" s="8">
         <f>V10-U10</f>
@@ -1441,7 +1441,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="S11" s="8">
         <f>R11-Q11</f>
@@ -1671,7 +1671,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="O13" s="8">
         <f>N13-L13</f>
@@ -1685,7 +1685,7 @@
         <v>0</v>
       </c>
       <c r="R13" s="8" t="n">
-        <v>942.8</v>
+        <v>628.53</v>
       </c>
       <c r="S13" s="8">
         <f>R13-Q13</f>
@@ -1699,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="8" t="n">
-        <v>166.9</v>
+        <v>111.27</v>
       </c>
       <c r="W13" s="8">
         <f>V13-U13</f>
@@ -1922,7 +1922,7 @@
         <v>13834961.34</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>32915174.69</v>
+        <v>31938287.19</v>
       </c>
       <c r="O15" s="8">
         <f>N15-L15</f>
@@ -1936,7 +1936,7 @@
         <v>18812341.93</v>
       </c>
       <c r="R15" s="8" t="n">
-        <v>27827753.11</v>
+        <v>25406547.17</v>
       </c>
       <c r="S15" s="8">
         <f>R15-Q15</f>
@@ -1950,7 +1950,7 @@
         <v>27342479.23</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>38013501.22</v>
+        <v>33214927.61</v>
       </c>
       <c r="W15" s="8">
         <f>V15-U15</f>
@@ -2044,7 +2044,7 @@
         <v>10111052.72</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>32638879.12</v>
+        <v>21137195.58</v>
       </c>
       <c r="O16" s="8">
         <f>N16-L16</f>
@@ -2058,7 +2058,7 @@
         <v>20693616.54</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>25887350.05</v>
+        <v>15671685.66</v>
       </c>
       <c r="S16" s="8">
         <f>R16-Q16</f>
@@ -2072,7 +2072,7 @@
         <v>25538510.67</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>34780251.58</v>
+        <v>19340819.95</v>
       </c>
       <c r="W16" s="8">
         <f>V16-U16</f>
@@ -2166,7 +2166,7 @@
         <v>10443752.94</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>23466512.89</v>
+        <v>21153775.33</v>
       </c>
       <c r="O17" s="8">
         <f>N17-L17</f>
@@ -2180,7 +2180,7 @@
         <v>13388655.95</v>
       </c>
       <c r="R17" s="8" t="n">
-        <v>19258898.38</v>
+        <v>12530409.78</v>
       </c>
       <c r="S17" s="8">
         <f>R17-Q17</f>
@@ -2194,7 +2194,7 @@
         <v>18892122.62</v>
       </c>
       <c r="V17" s="8" t="n">
-        <v>25776769.41</v>
+        <v>17681090.54</v>
       </c>
       <c r="W17" s="8">
         <f>V17-U17</f>
@@ -2288,7 +2288,7 @@
         <v>2451891.69</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>12119275.12</v>
+        <v>6216221.1</v>
       </c>
       <c r="O18" s="8">
         <f>N18-L18</f>
@@ -2302,7 +2302,7 @@
         <v>7021788.87</v>
       </c>
       <c r="R18" s="8" t="n">
-        <v>15016809.91</v>
+        <v>5908572.68</v>
       </c>
       <c r="S18" s="8">
         <f>R18-Q18</f>
@@ -2316,7 +2316,7 @@
         <v>7262073.52</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>17270461.46</v>
+        <v>6110763.22</v>
       </c>
       <c r="W18" s="8">
         <f>V18-U18</f>
@@ -2410,7 +2410,7 @@
         <v>3922507.01</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>9469497.439999999</v>
+        <v>9308085.529999999</v>
       </c>
       <c r="O19" s="8">
         <f>N19-L19</f>
@@ -2424,7 +2424,7 @@
         <v>6515033.17</v>
       </c>
       <c r="R19" s="8" t="n">
-        <v>8621598.800000001</v>
+        <v>8478180.859999999</v>
       </c>
       <c r="S19" s="8">
         <f>R19-Q19</f>
@@ -2438,7 +2438,7 @@
         <v>5125605.45</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>10172347.4</v>
+        <v>10146996.77</v>
       </c>
       <c r="W19" s="8">
         <f>V19-U19</f>
@@ -2532,7 +2532,7 @@
         <v>2067255.85</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>4122221.29</v>
+        <v>2845292.35</v>
       </c>
       <c r="O20" s="8">
         <f>N20-L20</f>
@@ -2546,7 +2546,7 @@
         <v>2909846.24</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>2785452.69</v>
+        <v>2292170.62</v>
       </c>
       <c r="S20" s="8">
         <f>R20-Q20</f>
@@ -2560,7 +2560,7 @@
         <v>2950894.62</v>
       </c>
       <c r="V20" s="8" t="n">
-        <v>4257657.02</v>
+        <v>3170581.1</v>
       </c>
       <c r="W20" s="8">
         <f>V20-U20</f>
@@ -2654,7 +2654,7 @@
         <v>2567043.91</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>3578646.12</v>
+        <v>3359320.03</v>
       </c>
       <c r="O21" s="8">
         <f>N21-L21</f>
@@ -2668,7 +2668,7 @@
         <v>1662305.66</v>
       </c>
       <c r="R21" s="8" t="n">
-        <v>3168644.1</v>
+        <v>2406211.14</v>
       </c>
       <c r="S21" s="8">
         <f>R21-Q21</f>
@@ -2682,7 +2682,7 @@
         <v>1567129.26</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>3019618.47</v>
+        <v>2182292.18</v>
       </c>
       <c r="W21" s="8">
         <f>V21-U21</f>
@@ -2790,7 +2790,7 @@
         <v>395145.64</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>612509.1800000001</v>
+        <v>612468.97</v>
       </c>
       <c r="S22" s="8">
         <f>R22-Q22</f>
@@ -2804,7 +2804,7 @@
         <v>411424.61</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>918703.46</v>
+        <v>612468.97</v>
       </c>
       <c r="W22" s="8">
         <f>V22-U22</f>
@@ -2898,7 +2898,7 @@
         <v>330988.56</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>747291.83</v>
+        <v>579944.78</v>
       </c>
       <c r="O23" s="8">
         <f>N23-L23</f>
@@ -2912,7 +2912,7 @@
         <v>335310.58</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>696636.59</v>
+        <v>557975.22</v>
       </c>
       <c r="S23" s="8">
         <f>R23-Q23</f>
@@ -2926,7 +2926,7 @@
         <v>395404.39</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>774765.66</v>
+        <v>572673.65</v>
       </c>
       <c r="W23" s="8">
         <f>V23-U23</f>
@@ -3020,7 +3020,7 @@
         <v>134647.24</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>411992.3</v>
+        <v>374874</v>
       </c>
       <c r="O24" s="8">
         <f>N24-L24</f>
@@ -3034,7 +3034,7 @@
         <v>241075.56</v>
       </c>
       <c r="R24" s="8" t="n">
-        <v>635901.8199999999</v>
+        <v>582269.26</v>
       </c>
       <c r="S24" s="8">
         <f>R24-Q24</f>
@@ -3048,7 +3048,7 @@
         <v>320808.69</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>608065.48</v>
+        <v>481042.03</v>
       </c>
       <c r="W24" s="8">
         <f>V24-U24</f>
@@ -3099,19 +3099,19 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>11452105</t>
+          <t>11452107</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>رسوم تراخيص حفر الشوارع</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>356658.1</v>
+        <v>1868556.75</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>1350</v>
+        <v>2750380.73</v>
       </c>
       <c r="F25" s="8">
         <f>E25-D25</f>
@@ -3122,10 +3122,10 @@
         <v/>
       </c>
       <c r="H25" s="8" t="n">
-        <v>31989.46</v>
+        <v>219460.02</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="J25" s="8">
         <f>I25-H25</f>
@@ -3136,13 +3136,13 @@
         <v/>
       </c>
       <c r="L25" s="8" t="n">
-        <v>32296.3</v>
+        <v>202820.15</v>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0</v>
+        <v>57100</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>2438320.04</v>
+        <v>57100</v>
       </c>
       <c r="O25" s="8">
         <f>N25-L25</f>
@@ -3153,10 +3153,10 @@
         <v/>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>27957.08</v>
+        <v>222880.38</v>
       </c>
       <c r="R25" s="8" t="n">
-        <v>1442670.34</v>
+        <v>10071.99</v>
       </c>
       <c r="S25" s="8">
         <f>R25-Q25</f>
@@ -3167,10 +3167,10 @@
         <v/>
       </c>
       <c r="U25" s="8" t="n">
-        <v>25146.7</v>
+        <v>327327.8</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>942302.9399999999</v>
+        <v>26903.01</v>
       </c>
       <c r="W25" s="8">
         <f>V25-U25</f>
@@ -3221,19 +3221,19 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>11452107</t>
+          <t>11452106</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>1868556.75</v>
+        <v>5585920.85</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>2750380.73</v>
+        <v>1363801.03</v>
       </c>
       <c r="F26" s="8">
         <f>E26-D26</f>
@@ -3244,10 +3244,10 @@
         <v/>
       </c>
       <c r="H26" s="8" t="n">
-        <v>219460.02</v>
+        <v>876071.65</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>32000</v>
+        <v>13800</v>
       </c>
       <c r="J26" s="8">
         <f>I26-H26</f>
@@ -3258,13 +3258,13 @@
         <v/>
       </c>
       <c r="L26" s="8" t="n">
-        <v>202820.15</v>
+        <v>759323.62</v>
       </c>
       <c r="M26" s="8" t="n">
-        <v>57100</v>
+        <v>56000</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>57100</v>
+        <v>56000</v>
       </c>
       <c r="O26" s="8">
         <f>N26-L26</f>
@@ -3275,10 +3275,10 @@
         <v/>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>222880.38</v>
+        <v>685167.54</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>15107.99</v>
+        <v>81304.39999999999</v>
       </c>
       <c r="S26" s="8">
         <f>R26-Q26</f>
@@ -3289,10 +3289,10 @@
         <v/>
       </c>
       <c r="U26" s="8" t="n">
-        <v>327327.8</v>
+        <v>572770.48</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>32025</v>
+        <v>81695.60000000001</v>
       </c>
       <c r="W26" s="8">
         <f>V26-U26</f>
@@ -3343,19 +3343,19 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>11452106</t>
+          <t>11452110</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>5585920.85</v>
+        <v>1035362.18</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>1363801.03</v>
+        <v>581755.84</v>
       </c>
       <c r="F27" s="8">
         <f>E27-D27</f>
@@ -3366,10 +3366,10 @@
         <v/>
       </c>
       <c r="H27" s="8" t="n">
-        <v>876071.65</v>
+        <v>151946.61</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>13800</v>
+        <v>20794.06</v>
       </c>
       <c r="J27" s="8">
         <f>I27-H27</f>
@@ -3380,13 +3380,13 @@
         <v/>
       </c>
       <c r="L27" s="8" t="n">
-        <v>759323.62</v>
+        <v>99448.75999999999</v>
       </c>
       <c r="M27" s="8" t="n">
-        <v>56000</v>
+        <v>34158.14</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>84000</v>
+        <v>37475.46</v>
       </c>
       <c r="O27" s="8">
         <f>N27-L27</f>
@@ -3397,10 +3397,10 @@
         <v/>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>685167.54</v>
+        <v>88463.77</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>121956.6</v>
+        <v>115379.71</v>
       </c>
       <c r="S27" s="8">
         <f>R27-Q27</f>
@@ -3411,10 +3411,10 @@
         <v/>
       </c>
       <c r="U27" s="8" t="n">
-        <v>572770.48</v>
+        <v>146186.3</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>122543.4</v>
+        <v>68083.02</v>
       </c>
       <c r="W27" s="8">
         <f>V27-U27</f>
@@ -3465,19 +3465,19 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>11452110</t>
+          <t>1422104</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+          <t>رسوم وأجور ناتجة من النشاط غير مصنفة أعلاه</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>1035362.18</v>
+        <v>0</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>581755.84</v>
+        <v>391830</v>
       </c>
       <c r="F28" s="8">
         <f>E28-D28</f>
@@ -3488,10 +3488,10 @@
         <v/>
       </c>
       <c r="H28" s="8" t="n">
-        <v>151946.61</v>
+        <v>0</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>20794.06</v>
+        <v>0</v>
       </c>
       <c r="J28" s="8">
         <f>I28-H28</f>
@@ -3502,13 +3502,13 @@
         <v/>
       </c>
       <c r="L28" s="8" t="n">
-        <v>99448.75999999999</v>
+        <v>0</v>
       </c>
       <c r="M28" s="8" t="n">
-        <v>34158.14</v>
+        <v>0</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>56213.19</v>
+        <v>0</v>
       </c>
       <c r="O28" s="8">
         <f>N28-L28</f>
@@ -3519,10 +3519,10 @@
         <v/>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>88463.77</v>
+        <v>0</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>115379.71</v>
+        <v>0</v>
       </c>
       <c r="S28" s="8">
         <f>R28-Q28</f>
@@ -3533,10 +3533,10 @@
         <v/>
       </c>
       <c r="U28" s="8" t="n">
-        <v>146186.3</v>
+        <v>0</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>82801.81</v>
+        <v>0</v>
       </c>
       <c r="W28" s="8">
         <f>V28-U28</f>
@@ -3587,19 +3587,19 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>1422104</t>
+          <t>11452109</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>رسوم وأجور ناتجة من النشاط غير مصنفة أعلاه</t>
+          <t>اعتماد مخططات التطوير العقاري</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>0</v>
+        <v>406632.44</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>391830</v>
+        <v>50</v>
       </c>
       <c r="F29" s="8">
         <f>E29-D29</f>
@@ -3610,7 +3610,7 @@
         <v/>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0</v>
+        <v>106451.02</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>0</v>
@@ -3624,13 +3624,13 @@
         <v/>
       </c>
       <c r="L29" s="8" t="n">
-        <v>0</v>
+        <v>212196.25</v>
       </c>
       <c r="M29" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>0</v>
+        <v>55147.96</v>
       </c>
       <c r="O29" s="8">
         <f>N29-L29</f>
@@ -3641,10 +3641,10 @@
         <v/>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0</v>
+        <v>49663.18</v>
       </c>
       <c r="R29" s="8" t="n">
-        <v>0</v>
+        <v>875.04</v>
       </c>
       <c r="S29" s="8">
         <f>R29-Q29</f>
@@ -3655,10 +3655,10 @@
         <v/>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0</v>
+        <v>185890.8</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0</v>
+        <v>2174.95</v>
       </c>
       <c r="W29" s="8">
         <f>V29-U29</f>
@@ -3709,19 +3709,19 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>11452109</t>
+          <t>1421907</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>اعتماد مخططات التطوير العقاري</t>
+          <t>إيرادات المخططات</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>406632.44</v>
+        <v>499531.96</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>50</v>
+        <v>5950</v>
       </c>
       <c r="F30" s="8">
         <f>E30-D30</f>
@@ -3732,7 +3732,7 @@
         <v/>
       </c>
       <c r="H30" s="8" t="n">
-        <v>106451.02</v>
+        <v>52413.24</v>
       </c>
       <c r="I30" s="8" t="n">
         <v>0</v>
@@ -3746,13 +3746,13 @@
         <v/>
       </c>
       <c r="L30" s="8" t="n">
-        <v>212196.25</v>
+        <v>55366.58</v>
       </c>
       <c r="M30" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>82721.94</v>
+        <v>0</v>
       </c>
       <c r="O30" s="8">
         <f>N30-L30</f>
@@ -3763,10 +3763,10 @@
         <v/>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>49663.18</v>
+        <v>32730.78</v>
       </c>
       <c r="R30" s="8" t="n">
-        <v>1312.57</v>
+        <v>0</v>
       </c>
       <c r="S30" s="8">
         <f>R30-Q30</f>
@@ -3777,10 +3777,10 @@
         <v/>
       </c>
       <c r="U30" s="8" t="n">
-        <v>185890.8</v>
+        <v>26407.51</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>3262.43</v>
+        <v>0</v>
       </c>
       <c r="W30" s="8">
         <f>V30-U30</f>
@@ -3831,19 +3831,19 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>1421907</t>
+          <t>11452513</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>إيرادات المخططات</t>
+          <t>لوحات إرشـادية</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>499531.96</v>
+        <v>47427</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>5950</v>
+        <v>600</v>
       </c>
       <c r="F31" s="8">
         <f>E31-D31</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="H31" s="8" t="n">
-        <v>52413.24</v>
+        <v>5106</v>
       </c>
       <c r="I31" s="8" t="n">
         <v>0</v>
@@ -3868,7 +3868,7 @@
         <v/>
       </c>
       <c r="L31" s="8" t="n">
-        <v>55366.58</v>
+        <v>5715</v>
       </c>
       <c r="M31" s="8" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v/>
       </c>
       <c r="Q31" s="8" t="n">
-        <v>32730.78</v>
+        <v>5723</v>
       </c>
       <c r="R31" s="8" t="n">
-        <v>0</v>
+        <v>649.95</v>
       </c>
       <c r="S31" s="8">
         <f>R31-Q31</f>
@@ -3899,10 +3899,10 @@
         <v/>
       </c>
       <c r="U31" s="8" t="n">
-        <v>26407.51</v>
+        <v>7794</v>
       </c>
       <c r="V31" s="8" t="n">
-        <v>0</v>
+        <v>400.05</v>
       </c>
       <c r="W31" s="8">
         <f>V31-U31</f>
@@ -3953,19 +3953,19 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>11452513</t>
+          <t>11452105</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>لوحات إرشـادية</t>
+          <t>رسوم تراخيص حفر الشوارع</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>47427</v>
+        <v>356658.1</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>600</v>
+        <v>1350</v>
       </c>
       <c r="F32" s="8">
         <f>E32-D32</f>
@@ -3976,7 +3976,7 @@
         <v/>
       </c>
       <c r="H32" s="8" t="n">
-        <v>5106</v>
+        <v>31989.46</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>0</v>
@@ -3990,7 +3990,7 @@
         <v/>
       </c>
       <c r="L32" s="8" t="n">
-        <v>5715</v>
+        <v>32296.3</v>
       </c>
       <c r="M32" s="8" t="n">
         <v>0</v>
@@ -4007,10 +4007,10 @@
         <v/>
       </c>
       <c r="Q32" s="8" t="n">
-        <v>5723</v>
+        <v>27957.08</v>
       </c>
       <c r="R32" s="8" t="n">
-        <v>974.9299999999999</v>
+        <v>0</v>
       </c>
       <c r="S32" s="8">
         <f>R32-Q32</f>
@@ -4021,10 +4021,10 @@
         <v/>
       </c>
       <c r="U32" s="8" t="n">
-        <v>7794</v>
+        <v>25146.7</v>
       </c>
       <c r="V32" s="8" t="n">
-        <v>600.08</v>
+        <v>0</v>
       </c>
       <c r="W32" s="8">
         <f>V32-U32</f>
@@ -4247,7 +4247,7 @@
         <v>33304429</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>48718919.41</v>
+        <v>44323914.15</v>
       </c>
       <c r="O34" s="8">
         <f>N34-L34</f>
@@ -4261,7 +4261,7 @@
         <v>28537922.26</v>
       </c>
       <c r="R34" s="8" t="n">
-        <v>41394654.55</v>
+        <v>39946977.27</v>
       </c>
       <c r="S34" s="8">
         <f>R34-Q34</f>
@@ -4275,7 +4275,7 @@
         <v>27405164.21</v>
       </c>
       <c r="V34" s="8" t="n">
-        <v>61541882.75</v>
+        <v>44453988.86</v>
       </c>
       <c r="W34" s="8">
         <f>V34-U34</f>
@@ -4383,7 +4383,7 @@
         <v>3380581.8</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>98690.73</v>
+        <v>65793.82000000001</v>
       </c>
       <c r="S35" s="8">
         <f>R35-Q35</f>
@@ -4397,7 +4397,7 @@
         <v>2982608.6</v>
       </c>
       <c r="V35" s="8" t="n">
-        <v>9570.27</v>
+        <v>6380.18</v>
       </c>
       <c r="W35" s="8">
         <f>V35-U35</f>
@@ -4613,7 +4613,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="O37" s="8">
         <f>N37-L37</f>
@@ -4627,7 +4627,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>17130.89</v>
+        <v>11420.59</v>
       </c>
       <c r="S37" s="8">
         <f>R37-Q37</f>
@@ -4641,7 +4641,7 @@
         <v>0</v>
       </c>
       <c r="V37" s="8" t="n">
-        <v>21794.11</v>
+        <v>14529.41</v>
       </c>
       <c r="W37" s="8">
         <f>V37-U37</f>
@@ -4864,7 +4864,7 @@
         <v>13283777.98</v>
       </c>
       <c r="N39" s="8" t="n">
-        <v>24243568.97</v>
+        <v>21389005.05</v>
       </c>
       <c r="O39" s="8">
         <f>N39-L39</f>
@@ -4878,7 +4878,7 @@
         <v>19850210.09</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>28572196.19</v>
+        <v>12959762.55</v>
       </c>
       <c r="S39" s="8">
         <f>R39-Q39</f>
@@ -4892,7 +4892,7 @@
         <v>23107944.17</v>
       </c>
       <c r="V39" s="8" t="n">
-        <v>26020979.2</v>
+        <v>15086664.99</v>
       </c>
       <c r="W39" s="8">
         <f>V39-U39</f>
@@ -4986,7 +4986,7 @@
         <v>3739768.97</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>7556764.42</v>
+        <v>5913098.76</v>
       </c>
       <c r="O40" s="8">
         <f>N40-L40</f>
@@ -5000,7 +5000,7 @@
         <v>5768559.67</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>7718698.21</v>
+        <v>4013782.75</v>
       </c>
       <c r="S40" s="8">
         <f>R40-Q40</f>
@@ -5014,7 +5014,7 @@
         <v>5209792.3</v>
       </c>
       <c r="V40" s="8" t="n">
-        <v>7281003.7</v>
+        <v>3624990.58</v>
       </c>
       <c r="W40" s="8">
         <f>V40-U40</f>
@@ -5108,7 +5108,7 @@
         <v>437434.24</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>2192443.14</v>
+        <v>893026.61</v>
       </c>
       <c r="O41" s="8">
         <f>N41-L41</f>
@@ -5122,7 +5122,7 @@
         <v>1246546.67</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>1854262.37</v>
+        <v>397672.58</v>
       </c>
       <c r="S41" s="8">
         <f>R41-Q41</f>
@@ -5136,7 +5136,7 @@
         <v>1183471.33</v>
       </c>
       <c r="V41" s="8" t="n">
-        <v>1865726.12</v>
+        <v>377550.32</v>
       </c>
       <c r="W41" s="8">
         <f>V41-U41</f>
@@ -5359,7 +5359,7 @@
         <v>7217587.27</v>
       </c>
       <c r="N43" s="8" t="n">
-        <v>14640342.46</v>
+        <v>8369863.23</v>
       </c>
       <c r="O43" s="8">
         <f>N43-L43</f>
@@ -5373,7 +5373,7 @@
         <v>2119658.52</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>8825433.380000001</v>
+        <v>7790081.04</v>
       </c>
       <c r="S43" s="8">
         <f>R43-Q43</f>
@@ -5387,7 +5387,7 @@
         <v>9129947.939999999</v>
       </c>
       <c r="V43" s="8" t="n">
-        <v>10106527.68</v>
+        <v>33554005.8</v>
       </c>
       <c r="W43" s="8">
         <f>V43-U43</f>
@@ -5481,7 +5481,7 @@
         <v>124953</v>
       </c>
       <c r="N44" s="8" t="n">
-        <v>1277426.25</v>
+        <v>851617.5</v>
       </c>
       <c r="O44" s="8">
         <f>N44-L44</f>
@@ -5495,7 +5495,7 @@
         <v>437120.39</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>333037.59</v>
+        <v>222025.06</v>
       </c>
       <c r="S44" s="8">
         <f>R44-Q44</f>
@@ -5509,7 +5509,7 @@
         <v>684676.76</v>
       </c>
       <c r="V44" s="8" t="n">
-        <v>338544.57</v>
+        <v>225696.38</v>
       </c>
       <c r="W44" s="8">
         <f>V44-U44</f>
@@ -5725,7 +5725,7 @@
         <v>179280.35</v>
       </c>
       <c r="N46" s="8" t="n">
-        <v>269650</v>
+        <v>212983.92</v>
       </c>
       <c r="O46" s="8">
         <f>N46-L46</f>
@@ -5739,7 +5739,7 @@
         <v>556377.2</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>270849</v>
+        <v>222778.16</v>
       </c>
       <c r="S46" s="8">
         <f>R46-Q46</f>
@@ -5753,7 +5753,7 @@
         <v>555958.98</v>
       </c>
       <c r="V46" s="8" t="n">
-        <v>196846.97</v>
+        <v>131231.31</v>
       </c>
       <c r="W46" s="8">
         <f>V46-U46</f>
@@ -5797,378 +5797,127 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>إجمالي علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="D47" s="5">
-        <f>SUM(D48:D48)</f>
-        <v/>
-      </c>
-      <c r="E47" s="5">
-        <f>SUM(E48:E48)</f>
-        <v/>
-      </c>
-      <c r="F47" s="5">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>الإجمالي العام</t>
+        </is>
+      </c>
+      <c r="D47" s="11">
+        <f>D6+D14+D33+D38+D42</f>
+        <v/>
+      </c>
+      <c r="E47" s="11">
+        <f>E6+E14+E33+E38+E42</f>
+        <v/>
+      </c>
+      <c r="F47" s="11">
         <f>E47-D47</f>
         <v/>
       </c>
-      <c r="G47" s="6">
+      <c r="G47" s="12">
         <f>IF(D47=0,"",E47/D47)</f>
         <v/>
       </c>
-      <c r="H47" s="5">
-        <f>SUM(H48:H48)</f>
-        <v/>
-      </c>
-      <c r="I47" s="5">
-        <f>SUM(I48:I48)</f>
-        <v/>
-      </c>
-      <c r="J47" s="5">
+      <c r="H47" s="11">
+        <f>H6+H14+H33+H38+H42</f>
+        <v/>
+      </c>
+      <c r="I47" s="11">
+        <f>I6+I14+I33+I38+I42</f>
+        <v/>
+      </c>
+      <c r="J47" s="11">
         <f>I47-H47</f>
         <v/>
       </c>
-      <c r="K47" s="6">
+      <c r="K47" s="12">
         <f>IF(H47=0,"",I47/H47)</f>
         <v/>
       </c>
-      <c r="L47" s="5">
-        <f>SUM(L48:L48)</f>
-        <v/>
-      </c>
-      <c r="M47" s="5">
-        <f>SUM(M48:M48)</f>
-        <v/>
-      </c>
-      <c r="N47" s="5">
-        <f>SUM(N48:N48)</f>
-        <v/>
-      </c>
-      <c r="O47" s="5">
+      <c r="L47" s="11">
+        <f>L6+L14+L33+L38+L42</f>
+        <v/>
+      </c>
+      <c r="M47" s="11">
+        <f>M6+M14+M33+M38+M42</f>
+        <v/>
+      </c>
+      <c r="N47" s="11">
+        <f>N6+N14+N33+N38+N42</f>
+        <v/>
+      </c>
+      <c r="O47" s="11">
         <f>N47-L47</f>
         <v/>
       </c>
-      <c r="P47" s="6">
+      <c r="P47" s="12">
         <f>IF(L47=0,"",N47/L47)</f>
         <v/>
       </c>
-      <c r="Q47" s="5">
-        <f>SUM(Q48:Q48)</f>
-        <v/>
-      </c>
-      <c r="R47" s="5">
-        <f>SUM(R48:R48)</f>
-        <v/>
-      </c>
-      <c r="S47" s="5">
+      <c r="Q47" s="11">
+        <f>Q6+Q14+Q33+Q38+Q42</f>
+        <v/>
+      </c>
+      <c r="R47" s="11">
+        <f>R6+R14+R33+R38+R42</f>
+        <v/>
+      </c>
+      <c r="S47" s="11">
         <f>R47-Q47</f>
         <v/>
       </c>
-      <c r="T47" s="6">
+      <c r="T47" s="12">
         <f>IF(Q47=0,"",R47/Q47)</f>
         <v/>
       </c>
-      <c r="U47" s="5">
-        <f>SUM(U48:U48)</f>
-        <v/>
-      </c>
-      <c r="V47" s="5">
-        <f>SUM(V48:V48)</f>
-        <v/>
-      </c>
-      <c r="W47" s="5">
+      <c r="U47" s="11">
+        <f>U6+U14+U33+U38+U42</f>
+        <v/>
+      </c>
+      <c r="V47" s="11">
+        <f>V6+V14+V33+V38+V42</f>
+        <v/>
+      </c>
+      <c r="W47" s="11">
         <f>V47-U47</f>
         <v/>
       </c>
-      <c r="X47" s="6">
+      <c r="X47" s="12">
         <f>IF(U47=0,"",V47/U47)</f>
         <v/>
       </c>
-      <c r="Y47" s="5">
+      <c r="Y47" s="11">
         <f>L47+Q47+U47</f>
         <v/>
       </c>
-      <c r="Z47" s="5">
+      <c r="Z47" s="11">
         <f>N47+R47+V47</f>
         <v/>
       </c>
-      <c r="AA47" s="5">
+      <c r="AA47" s="11">
         <f>Z47-Y47</f>
         <v/>
       </c>
-      <c r="AB47" s="6">
+      <c r="AB47" s="12">
         <f>IF(Y47=0,"",Z47/Y47)</f>
         <v/>
       </c>
-      <c r="AC47" s="5">
+      <c r="AC47" s="11">
         <f>D47+Y47</f>
         <v/>
       </c>
-      <c r="AD47" s="5">
+      <c r="AD47" s="11">
         <f>E47+Z47</f>
         <v/>
       </c>
-      <c r="AE47" s="5">
+      <c r="AE47" s="11">
         <f>AD47-AC47</f>
         <v/>
       </c>
-      <c r="AF47" s="6">
+      <c r="AF47" s="12">
         <f>IF(AC47=0,"",AD47/AC47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>بدون رقم</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>بدون رقم (خدمات علم + جزاءات)</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="8">
-        <f>E48-D48</f>
-        <v/>
-      </c>
-      <c r="G48" s="9">
-        <f>IF(D48=0,"",E48/D48)</f>
-        <v/>
-      </c>
-      <c r="H48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="8">
-        <f>I48-H48</f>
-        <v/>
-      </c>
-      <c r="K48" s="9">
-        <f>IF(H48=0,"",I48/H48)</f>
-        <v/>
-      </c>
-      <c r="L48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" s="8" t="n">
-        <v>390906.25</v>
-      </c>
-      <c r="N48" s="8" t="n">
-        <v>1246768.12</v>
-      </c>
-      <c r="O48" s="8">
-        <f>N48-L48</f>
-        <v/>
-      </c>
-      <c r="P48" s="9">
-        <f>IF(L48=0,"",N48/L48)</f>
-        <v/>
-      </c>
-      <c r="Q48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" s="8" t="n">
-        <v>1133123.14</v>
-      </c>
-      <c r="S48" s="8">
-        <f>R48-Q48</f>
-        <v/>
-      </c>
-      <c r="T48" s="9">
-        <f>IF(Q48=0,"",R48/Q48)</f>
-        <v/>
-      </c>
-      <c r="U48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V48" s="8" t="n">
-        <v>1216779.68</v>
-      </c>
-      <c r="W48" s="8">
-        <f>V48-U48</f>
-        <v/>
-      </c>
-      <c r="X48" s="9">
-        <f>IF(U48=0,"",V48/U48)</f>
-        <v/>
-      </c>
-      <c r="Y48" s="8">
-        <f>L48+Q48+U48</f>
-        <v/>
-      </c>
-      <c r="Z48" s="8">
-        <f>N48+R48+V48</f>
-        <v/>
-      </c>
-      <c r="AA48" s="8">
-        <f>Z48-Y48</f>
-        <v/>
-      </c>
-      <c r="AB48" s="9">
-        <f>IF(Y48=0,"",Z48/Y48)</f>
-        <v/>
-      </c>
-      <c r="AC48" s="8">
-        <f>D48+Y48</f>
-        <v/>
-      </c>
-      <c r="AD48" s="8">
-        <f>E48+Z48</f>
-        <v/>
-      </c>
-      <c r="AE48" s="8">
-        <f>AD48-AC48</f>
-        <v/>
-      </c>
-      <c r="AF48" s="9">
-        <f>IF(AC48=0,"",AD48/AC48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="n"/>
-      <c r="B49" s="10" t="n"/>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>الإجمالي العام</t>
-        </is>
-      </c>
-      <c r="D49" s="11">
-        <f>D6+D14+D33+D38+D42+D47</f>
-        <v/>
-      </c>
-      <c r="E49" s="11">
-        <f>E6+E14+E33+E38+E42+E47</f>
-        <v/>
-      </c>
-      <c r="F49" s="11">
-        <f>E49-D49</f>
-        <v/>
-      </c>
-      <c r="G49" s="12">
-        <f>IF(D49=0,"",E49/D49)</f>
-        <v/>
-      </c>
-      <c r="H49" s="11">
-        <f>H6+H14+H33+H38+H42+H47</f>
-        <v/>
-      </c>
-      <c r="I49" s="11">
-        <f>I6+I14+I33+I38+I42+I47</f>
-        <v/>
-      </c>
-      <c r="J49" s="11">
-        <f>I49-H49</f>
-        <v/>
-      </c>
-      <c r="K49" s="12">
-        <f>IF(H49=0,"",I49/H49)</f>
-        <v/>
-      </c>
-      <c r="L49" s="11">
-        <f>L6+L14+L33+L38+L42+L47</f>
-        <v/>
-      </c>
-      <c r="M49" s="11">
-        <f>M6+M14+M33+M38+M42+M47</f>
-        <v/>
-      </c>
-      <c r="N49" s="11">
-        <f>N6+N14+N33+N38+N42+N47</f>
-        <v/>
-      </c>
-      <c r="O49" s="11">
-        <f>N49-L49</f>
-        <v/>
-      </c>
-      <c r="P49" s="12">
-        <f>IF(L49=0,"",N49/L49)</f>
-        <v/>
-      </c>
-      <c r="Q49" s="11">
-        <f>Q6+Q14+Q33+Q38+Q42+Q47</f>
-        <v/>
-      </c>
-      <c r="R49" s="11">
-        <f>R6+R14+R33+R38+R42+R47</f>
-        <v/>
-      </c>
-      <c r="S49" s="11">
-        <f>R49-Q49</f>
-        <v/>
-      </c>
-      <c r="T49" s="12">
-        <f>IF(Q49=0,"",R49/Q49)</f>
-        <v/>
-      </c>
-      <c r="U49" s="11">
-        <f>U6+U14+U33+U38+U42+U47</f>
-        <v/>
-      </c>
-      <c r="V49" s="11">
-        <f>V6+V14+V33+V38+V42+V47</f>
-        <v/>
-      </c>
-      <c r="W49" s="11">
-        <f>V49-U49</f>
-        <v/>
-      </c>
-      <c r="X49" s="12">
-        <f>IF(U49=0,"",V49/U49)</f>
-        <v/>
-      </c>
-      <c r="Y49" s="11">
-        <f>L49+Q49+U49</f>
-        <v/>
-      </c>
-      <c r="Z49" s="11">
-        <f>N49+R49+V49</f>
-        <v/>
-      </c>
-      <c r="AA49" s="11">
-        <f>Z49-Y49</f>
-        <v/>
-      </c>
-      <c r="AB49" s="12">
-        <f>IF(Y49=0,"",Z49/Y49)</f>
-        <v/>
-      </c>
-      <c r="AC49" s="11">
-        <f>D49+Y49</f>
-        <v/>
-      </c>
-      <c r="AD49" s="11">
-        <f>E49+Z49</f>
-        <v/>
-      </c>
-      <c r="AE49" s="11">
-        <f>AD49-AC49</f>
-        <v/>
-      </c>
-      <c r="AF49" s="12">
-        <f>IF(AC49=0,"",AD49/AC49)</f>
         <v/>
       </c>
     </row>
@@ -6196,7 +5945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF49"/>
+  <dimension ref="A1:AF47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6236,14 +5985,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل التراكمي حتى سبتمبر والشهري سبتمبر–ديسمبر 2026 — الأسوأ (متحفظ)</t>
+          <t>المستهدف والمحصل التراكمي حتى سبتمبر والشهري سبتمبر–ديسمبر 2026 — الأسوأ (أرقامك المعدّلة)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. طريقة الأسوأ: لكل شهر، أدنى قيمة تاريخية لنفس الشهر (2023–2025) × معامل الاتجاه (بحد أقصى 1)، ولا يقل أكتوبر عن المحصل حتى تاريخه.</t>
+          <t>المستهدف والمحصل الفعلي من ملف المراقبة (قبل الاستقطاع، بدون ضريبة القيمة المضافة). التراكمي = مجموع يناير إلى سبتمبر، وسبتمبر مشمول فيه ويُعرض منفصلاً للتوضيح فقط (لا يُجمع مع التراكمي). إجمالي السنة = التراكمي + أكتوبر + نوفمبر + ديسمبر، ومجموع المستهدف السنوي 4,050 مليون يطابق ملف المراقبة. أكتوبر: المحصل حتى تاريخ الملف مع توقع الشهر كاملاً. نوفمبر وديسمبر: توقع. الأرقام بالريال والحسابات مجمّعة تحت التبويب. الأسوأ = عمود "إقفال 2026 – أسوأ" في ملفك المعدّل لكل حساب. للحسابات التي عدّلتها وُزّع الباقي على بقية أكتوبر ونوفمبر وديسمبر بنسب المستهدف الشهري للحساب؛ وغيرها بقي على توزيع الأسوأ (أدنى قيمة تاريخية لكل شهر × الاتجاه بحد أقصى 1). لا ينزل أي حساب عن المحصل الفعلي.</t>
         </is>
       </c>
     </row>
@@ -10576,7 +10325,7 @@
         <v>13283777.98</v>
       </c>
       <c r="N39" s="8" t="n">
-        <v>13283777.98</v>
+        <v>17437181.24</v>
       </c>
       <c r="O39" s="8">
         <f>N39-L39</f>
@@ -10590,7 +10339,7 @@
         <v>19850210.09</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>21246746.31</v>
+        <v>6641037.89</v>
       </c>
       <c r="S39" s="8">
         <f>R39-Q39</f>
@@ -10604,7 +10353,7 @@
         <v>23107944.17</v>
       </c>
       <c r="V39" s="8" t="n">
-        <v>17278632.31</v>
+        <v>7730937.46</v>
       </c>
       <c r="W39" s="8">
         <f>V39-U39</f>
@@ -10698,7 +10447,7 @@
         <v>3739768.97</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>4881210.37</v>
+        <v>4775658.74</v>
       </c>
       <c r="O40" s="8">
         <f>N40-L40</f>
@@ -10712,7 +10461,7 @@
         <v>5768559.67</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>5248722.33</v>
+        <v>1913118.08</v>
       </c>
       <c r="S40" s="8">
         <f>R40-Q40</f>
@@ -10726,7 +10475,7 @@
         <v>5209792.3</v>
       </c>
       <c r="V40" s="8" t="n">
-        <v>5286649.66</v>
+        <v>1727805.27</v>
       </c>
       <c r="W40" s="8">
         <f>V40-U40</f>
@@ -10820,7 +10569,7 @@
         <v>437434.24</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>973250</v>
+        <v>893026.61</v>
       </c>
       <c r="O41" s="8">
         <f>N41-L41</f>
@@ -10834,7 +10583,7 @@
         <v>1246546.67</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>1295756</v>
+        <v>397672.58</v>
       </c>
       <c r="S41" s="8">
         <f>R41-Q41</f>
@@ -10848,7 +10597,7 @@
         <v>1183471.33</v>
       </c>
       <c r="V41" s="8" t="n">
-        <v>1399244</v>
+        <v>377550.32</v>
       </c>
       <c r="W41" s="8">
         <f>V41-U41</f>
@@ -11071,7 +10820,7 @@
         <v>7217587.27</v>
       </c>
       <c r="N43" s="8" t="n">
-        <v>7217587.27</v>
+        <v>8369863.23</v>
       </c>
       <c r="O43" s="8">
         <f>N43-L43</f>
@@ -11085,7 +10834,7 @@
         <v>2119658.52</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>1161058.18</v>
+        <v>7790081.04</v>
       </c>
       <c r="S43" s="8">
         <f>R43-Q43</f>
@@ -11099,7 +10848,7 @@
         <v>9129947.939999999</v>
       </c>
       <c r="V43" s="8" t="n">
-        <v>1335304.27</v>
+        <v>33554005.8</v>
       </c>
       <c r="W43" s="8">
         <f>V43-U43</f>
@@ -11509,378 +11258,127 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>إجمالي علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="D47" s="5">
-        <f>SUM(D48:D48)</f>
-        <v/>
-      </c>
-      <c r="E47" s="5">
-        <f>SUM(E48:E48)</f>
-        <v/>
-      </c>
-      <c r="F47" s="5">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>الإجمالي العام</t>
+        </is>
+      </c>
+      <c r="D47" s="11">
+        <f>D6+D14+D33+D38+D42</f>
+        <v/>
+      </c>
+      <c r="E47" s="11">
+        <f>E6+E14+E33+E38+E42</f>
+        <v/>
+      </c>
+      <c r="F47" s="11">
         <f>E47-D47</f>
         <v/>
       </c>
-      <c r="G47" s="6">
+      <c r="G47" s="12">
         <f>IF(D47=0,"",E47/D47)</f>
         <v/>
       </c>
-      <c r="H47" s="5">
-        <f>SUM(H48:H48)</f>
-        <v/>
-      </c>
-      <c r="I47" s="5">
-        <f>SUM(I48:I48)</f>
-        <v/>
-      </c>
-      <c r="J47" s="5">
+      <c r="H47" s="11">
+        <f>H6+H14+H33+H38+H42</f>
+        <v/>
+      </c>
+      <c r="I47" s="11">
+        <f>I6+I14+I33+I38+I42</f>
+        <v/>
+      </c>
+      <c r="J47" s="11">
         <f>I47-H47</f>
         <v/>
       </c>
-      <c r="K47" s="6">
+      <c r="K47" s="12">
         <f>IF(H47=0,"",I47/H47)</f>
         <v/>
       </c>
-      <c r="L47" s="5">
-        <f>SUM(L48:L48)</f>
-        <v/>
-      </c>
-      <c r="M47" s="5">
-        <f>SUM(M48:M48)</f>
-        <v/>
-      </c>
-      <c r="N47" s="5">
-        <f>SUM(N48:N48)</f>
-        <v/>
-      </c>
-      <c r="O47" s="5">
+      <c r="L47" s="11">
+        <f>L6+L14+L33+L38+L42</f>
+        <v/>
+      </c>
+      <c r="M47" s="11">
+        <f>M6+M14+M33+M38+M42</f>
+        <v/>
+      </c>
+      <c r="N47" s="11">
+        <f>N6+N14+N33+N38+N42</f>
+        <v/>
+      </c>
+      <c r="O47" s="11">
         <f>N47-L47</f>
         <v/>
       </c>
-      <c r="P47" s="6">
+      <c r="P47" s="12">
         <f>IF(L47=0,"",N47/L47)</f>
         <v/>
       </c>
-      <c r="Q47" s="5">
-        <f>SUM(Q48:Q48)</f>
-        <v/>
-      </c>
-      <c r="R47" s="5">
-        <f>SUM(R48:R48)</f>
-        <v/>
-      </c>
-      <c r="S47" s="5">
+      <c r="Q47" s="11">
+        <f>Q6+Q14+Q33+Q38+Q42</f>
+        <v/>
+      </c>
+      <c r="R47" s="11">
+        <f>R6+R14+R33+R38+R42</f>
+        <v/>
+      </c>
+      <c r="S47" s="11">
         <f>R47-Q47</f>
         <v/>
       </c>
-      <c r="T47" s="6">
+      <c r="T47" s="12">
         <f>IF(Q47=0,"",R47/Q47)</f>
         <v/>
       </c>
-      <c r="U47" s="5">
-        <f>SUM(U48:U48)</f>
-        <v/>
-      </c>
-      <c r="V47" s="5">
-        <f>SUM(V48:V48)</f>
-        <v/>
-      </c>
-      <c r="W47" s="5">
+      <c r="U47" s="11">
+        <f>U6+U14+U33+U38+U42</f>
+        <v/>
+      </c>
+      <c r="V47" s="11">
+        <f>V6+V14+V33+V38+V42</f>
+        <v/>
+      </c>
+      <c r="W47" s="11">
         <f>V47-U47</f>
         <v/>
       </c>
-      <c r="X47" s="6">
+      <c r="X47" s="12">
         <f>IF(U47=0,"",V47/U47)</f>
         <v/>
       </c>
-      <c r="Y47" s="5">
+      <c r="Y47" s="11">
         <f>L47+Q47+U47</f>
         <v/>
       </c>
-      <c r="Z47" s="5">
+      <c r="Z47" s="11">
         <f>N47+R47+V47</f>
         <v/>
       </c>
-      <c r="AA47" s="5">
+      <c r="AA47" s="11">
         <f>Z47-Y47</f>
         <v/>
       </c>
-      <c r="AB47" s="6">
+      <c r="AB47" s="12">
         <f>IF(Y47=0,"",Z47/Y47)</f>
         <v/>
       </c>
-      <c r="AC47" s="5">
+      <c r="AC47" s="11">
         <f>D47+Y47</f>
         <v/>
       </c>
-      <c r="AD47" s="5">
+      <c r="AD47" s="11">
         <f>E47+Z47</f>
         <v/>
       </c>
-      <c r="AE47" s="5">
+      <c r="AE47" s="11">
         <f>AD47-AC47</f>
         <v/>
       </c>
-      <c r="AF47" s="6">
+      <c r="AF47" s="12">
         <f>IF(AC47=0,"",AD47/AC47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>بدون رقم</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>بدون رقم (خدمات علم + جزاءات)</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="8">
-        <f>E48-D48</f>
-        <v/>
-      </c>
-      <c r="G48" s="9">
-        <f>IF(D48=0,"",E48/D48)</f>
-        <v/>
-      </c>
-      <c r="H48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="8">
-        <f>I48-H48</f>
-        <v/>
-      </c>
-      <c r="K48" s="9">
-        <f>IF(H48=0,"",I48/H48)</f>
-        <v/>
-      </c>
-      <c r="L48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" s="8" t="n">
-        <v>390906.25</v>
-      </c>
-      <c r="N48" s="8" t="n">
-        <v>390906.25</v>
-      </c>
-      <c r="O48" s="8">
-        <f>N48-L48</f>
-        <v/>
-      </c>
-      <c r="P48" s="9">
-        <f>IF(L48=0,"",N48/L48)</f>
-        <v/>
-      </c>
-      <c r="Q48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" s="8" t="n">
-        <v>264165.43</v>
-      </c>
-      <c r="S48" s="8">
-        <f>R48-Q48</f>
-        <v/>
-      </c>
-      <c r="T48" s="9">
-        <f>IF(Q48=0,"",R48/Q48)</f>
-        <v/>
-      </c>
-      <c r="U48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V48" s="8" t="n">
-        <v>283668.32</v>
-      </c>
-      <c r="W48" s="8">
-        <f>V48-U48</f>
-        <v/>
-      </c>
-      <c r="X48" s="9">
-        <f>IF(U48=0,"",V48/U48)</f>
-        <v/>
-      </c>
-      <c r="Y48" s="8">
-        <f>L48+Q48+U48</f>
-        <v/>
-      </c>
-      <c r="Z48" s="8">
-        <f>N48+R48+V48</f>
-        <v/>
-      </c>
-      <c r="AA48" s="8">
-        <f>Z48-Y48</f>
-        <v/>
-      </c>
-      <c r="AB48" s="9">
-        <f>IF(Y48=0,"",Z48/Y48)</f>
-        <v/>
-      </c>
-      <c r="AC48" s="8">
-        <f>D48+Y48</f>
-        <v/>
-      </c>
-      <c r="AD48" s="8">
-        <f>E48+Z48</f>
-        <v/>
-      </c>
-      <c r="AE48" s="8">
-        <f>AD48-AC48</f>
-        <v/>
-      </c>
-      <c r="AF48" s="9">
-        <f>IF(AC48=0,"",AD48/AC48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="n"/>
-      <c r="B49" s="10" t="n"/>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>الإجمالي العام</t>
-        </is>
-      </c>
-      <c r="D49" s="11">
-        <f>D6+D14+D33+D38+D42+D47</f>
-        <v/>
-      </c>
-      <c r="E49" s="11">
-        <f>E6+E14+E33+E38+E42+E47</f>
-        <v/>
-      </c>
-      <c r="F49" s="11">
-        <f>E49-D49</f>
-        <v/>
-      </c>
-      <c r="G49" s="12">
-        <f>IF(D49=0,"",E49/D49)</f>
-        <v/>
-      </c>
-      <c r="H49" s="11">
-        <f>H6+H14+H33+H38+H42+H47</f>
-        <v/>
-      </c>
-      <c r="I49" s="11">
-        <f>I6+I14+I33+I38+I42+I47</f>
-        <v/>
-      </c>
-      <c r="J49" s="11">
-        <f>I49-H49</f>
-        <v/>
-      </c>
-      <c r="K49" s="12">
-        <f>IF(H49=0,"",I49/H49)</f>
-        <v/>
-      </c>
-      <c r="L49" s="11">
-        <f>L6+L14+L33+L38+L42+L47</f>
-        <v/>
-      </c>
-      <c r="M49" s="11">
-        <f>M6+M14+M33+M38+M42+M47</f>
-        <v/>
-      </c>
-      <c r="N49" s="11">
-        <f>N6+N14+N33+N38+N42+N47</f>
-        <v/>
-      </c>
-      <c r="O49" s="11">
-        <f>N49-L49</f>
-        <v/>
-      </c>
-      <c r="P49" s="12">
-        <f>IF(L49=0,"",N49/L49)</f>
-        <v/>
-      </c>
-      <c r="Q49" s="11">
-        <f>Q6+Q14+Q33+Q38+Q42+Q47</f>
-        <v/>
-      </c>
-      <c r="R49" s="11">
-        <f>R6+R14+R33+R38+R42+R47</f>
-        <v/>
-      </c>
-      <c r="S49" s="11">
-        <f>R49-Q49</f>
-        <v/>
-      </c>
-      <c r="T49" s="12">
-        <f>IF(Q49=0,"",R49/Q49)</f>
-        <v/>
-      </c>
-      <c r="U49" s="11">
-        <f>U6+U14+U33+U38+U42+U47</f>
-        <v/>
-      </c>
-      <c r="V49" s="11">
-        <f>V6+V14+V33+V38+V42+V47</f>
-        <v/>
-      </c>
-      <c r="W49" s="11">
-        <f>V49-U49</f>
-        <v/>
-      </c>
-      <c r="X49" s="12">
-        <f>IF(U49=0,"",V49/U49)</f>
-        <v/>
-      </c>
-      <c r="Y49" s="11">
-        <f>L49+Q49+U49</f>
-        <v/>
-      </c>
-      <c r="Z49" s="11">
-        <f>N49+R49+V49</f>
-        <v/>
-      </c>
-      <c r="AA49" s="11">
-        <f>Z49-Y49</f>
-        <v/>
-      </c>
-      <c r="AB49" s="12">
-        <f>IF(Y49=0,"",Z49/Y49)</f>
-        <v/>
-      </c>
-      <c r="AC49" s="11">
-        <f>D49+Y49</f>
-        <v/>
-      </c>
-      <c r="AD49" s="11">
-        <f>E49+Z49</f>
-        <v/>
-      </c>
-      <c r="AE49" s="11">
-        <f>AD49-AC49</f>
-        <v/>
-      </c>
-      <c r="AF49" s="12">
-        <f>IF(AC49=0,"",AD49/AC49)</f>
         <v/>
       </c>
     </row>

</xml_diff>